<commit_message>
redoing phylogenies and making the figure look nicer
</commit_message>
<xml_diff>
--- a/data/01_pd-samples/26_01_15_pd_samples-edited.xlsx
+++ b/data/01_pd-samples/26_01_15_pd_samples-edited.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/caprinapugliese/Documents/03_school/Uconn/2024-26_Grad_School/Dagilis-lab/WNS-project/data/01_pd-samples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D74F1B-FB60-E04C-9E0C-8E42BCDB93E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68EDBDDA-3160-7947-902B-79468568869F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14440" yWindow="22100" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{D99E271A-162C-F24C-8D0E-BBA6ED327C07}"/>
+    <workbookView xWindow="6920" yWindow="2480" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{D99E271A-162C-F24C-8D0E-BBA6ED327C07}"/>
   </bookViews>
   <sheets>
     <sheet name="25_10-16_pd_samples-edited" sheetId="1" r:id="rId1"/>
@@ -1890,7 +1890,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1947,7 +1947,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2078,7 +2077,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{18C33721-6494-9A49-9427-66EBEE919E8D}" name="Table14" displayName="Table14" ref="A1:Y68" totalsRowShown="0">
   <autoFilter ref="A1:Y68" xr:uid="{90C14361-2949-B74A-BFF6-1CEFD0790204}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Y68">
-    <sortCondition descending="1" ref="M1:M68"/>
+    <sortCondition ref="B1:B68"/>
   </sortState>
   <tableColumns count="25">
     <tableColumn id="1" xr3:uid="{B94284E2-80D9-FD40-B6D3-31E24510FDA8}" name="sample_id"/>
@@ -7023,25 +7022,25 @@
     </row>
     <row r="2" spans="1:25" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>150</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>234</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>150</v>
+        <v>13</v>
       </c>
       <c r="D2" s="5">
-        <v>6011486</v>
+        <v>3545531</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>235</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>232</v>
+        <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>233</v>
+        <v>17</v>
       </c>
       <c r="H2">
         <v>2016</v>
@@ -7050,435 +7049,495 @@
         <v>2016</v>
       </c>
       <c r="J2" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="K2" t="s">
-        <v>43</v>
-      </c>
-      <c r="L2" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="M2" s="32" t="s">
-        <v>428</v>
+        <v>19</v>
+      </c>
+      <c r="L2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" s="7" t="s">
+        <v>305</v>
       </c>
       <c r="N2" t="s">
-        <v>237</v>
+        <v>298</v>
       </c>
       <c r="O2" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="P2" t="s">
-        <v>237</v>
-      </c>
-      <c r="R2">
-        <v>46.823079999999997</v>
-      </c>
-      <c r="S2">
-        <v>102.503703</v>
+        <v>309</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>406</v>
+      </c>
+      <c r="R2" s="8">
+        <v>43.0274</v>
+      </c>
+      <c r="S2" s="8">
+        <v>-90.092200000000005</v>
+      </c>
+      <c r="X2" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>409</v>
       </c>
     </row>
     <row r="3" spans="1:25" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>122</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>123</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s">
-        <v>122</v>
+        <v>21</v>
       </c>
       <c r="D3" s="5">
-        <v>1952982</v>
+        <v>3411506</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>124</v>
+        <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="G3" t="s">
-        <v>125</v>
+        <v>24</v>
       </c>
       <c r="H3">
-        <v>2008</v>
+        <v>2010</v>
       </c>
       <c r="I3">
-        <v>2008</v>
+        <v>2010</v>
       </c>
       <c r="J3" t="s">
-        <v>117</v>
+        <v>18</v>
       </c>
       <c r="K3" t="s">
-        <v>43</v>
-      </c>
-      <c r="L3" t="s">
-        <v>20</v>
-      </c>
-      <c r="M3" t="s">
-        <v>427</v>
+        <v>19</v>
+      </c>
+      <c r="L3" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>305</v>
       </c>
       <c r="N3" t="s">
-        <v>298</v>
+        <v>314</v>
       </c>
       <c r="O3" t="s">
-        <v>299</v>
+        <v>315</v>
       </c>
       <c r="P3" t="s">
-        <v>328</v>
+        <v>316</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>402</v>
       </c>
       <c r="R3">
-        <v>41.844515371877698</v>
+        <v>49.954439999999998</v>
       </c>
       <c r="S3">
-        <v>-74.098548155198898</v>
-      </c>
-      <c r="T3" t="s">
-        <v>379</v>
-      </c>
-      <c r="U3" t="s">
-        <v>380</v>
+        <v>14.175829999999999</v>
       </c>
       <c r="V3" t="s">
-        <v>378</v>
+        <v>403</v>
       </c>
       <c r="W3" t="s">
-        <v>384</v>
-      </c>
-      <c r="X3" s="6" t="s">
-        <v>386</v>
-      </c>
-      <c r="Y3" s="2" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
+        <v>401</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" ht="51" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>168</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>169</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>168</v>
+        <v>27</v>
       </c>
       <c r="D4" s="5">
-        <v>6011467</v>
+        <v>3411507</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>170</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="G4" t="s">
-        <v>171</v>
+        <v>30</v>
       </c>
       <c r="H4">
-        <v>2009</v>
-      </c>
-      <c r="I4" s="1">
-        <v>39879</v>
+        <v>2010</v>
+      </c>
+      <c r="I4">
+        <v>2010</v>
       </c>
       <c r="J4" t="s">
-        <v>130</v>
+        <v>18</v>
       </c>
       <c r="K4" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="L4" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="M4" s="32" t="s">
-        <v>427</v>
+      <c r="M4" s="7" t="s">
+        <v>305</v>
       </c>
       <c r="N4" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="O4" t="s">
-        <v>324</v>
+        <v>315</v>
       </c>
       <c r="P4" t="s">
-        <v>305</v>
+        <v>316</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>402</v>
       </c>
       <c r="R4">
-        <v>50.788476564399403</v>
+        <v>49.954439999999998</v>
       </c>
       <c r="S4">
-        <v>10.740499703414899</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
+        <v>14.175829999999999</v>
+      </c>
+      <c r="V4" t="s">
+        <v>403</v>
+      </c>
+      <c r="W4" t="s">
+        <v>17</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>171</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>172</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>171</v>
+        <v>31</v>
       </c>
       <c r="D5" s="5">
-        <v>6011468</v>
+        <v>3411508</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>173</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="G5" t="s">
-        <v>174</v>
+        <v>34</v>
       </c>
       <c r="H5">
-        <v>2009</v>
-      </c>
-      <c r="I5" s="1">
-        <v>39904</v>
+        <v>2011</v>
+      </c>
+      <c r="I5">
+        <v>2011</v>
       </c>
       <c r="J5" t="s">
-        <v>130</v>
+        <v>18</v>
       </c>
       <c r="K5" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="L5" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="M5" s="32" t="s">
-        <v>427</v>
+      <c r="M5" s="7" t="s">
+        <v>305</v>
       </c>
       <c r="N5" t="s">
-        <v>336</v>
+        <v>314</v>
       </c>
       <c r="O5" t="s">
-        <v>338</v>
+        <v>317</v>
       </c>
       <c r="P5" t="s">
-        <v>305</v>
+        <v>318</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>402</v>
       </c>
       <c r="R5">
-        <v>47.083329999999997</v>
+        <v>50.693460000000002</v>
       </c>
       <c r="S5">
-        <v>8</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>26</v>
+        <v>15.84652</v>
+      </c>
+      <c r="V5" t="s">
+        <v>405</v>
+      </c>
+      <c r="W5" t="s">
+        <v>24</v>
+      </c>
+      <c r="X5" s="6" t="s">
+        <v>400</v>
       </c>
     </row>
     <row r="6" spans="1:25" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>209</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>210</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>209</v>
+        <v>35</v>
       </c>
       <c r="D6" s="5">
-        <v>6011465</v>
+        <v>3411509</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>211</v>
+        <v>37</v>
       </c>
       <c r="F6" t="s">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="G6" t="s">
-        <v>212</v>
+        <v>13</v>
       </c>
       <c r="H6">
-        <v>2009</v>
-      </c>
-      <c r="I6" s="1">
-        <v>39901</v>
+        <v>2011</v>
+      </c>
+      <c r="I6">
+        <v>2011</v>
       </c>
       <c r="J6" t="s">
-        <v>130</v>
+        <v>18</v>
       </c>
       <c r="K6" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="L6" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="32" t="s">
-        <v>427</v>
+      <c r="M6" s="7" t="s">
+        <v>305</v>
       </c>
       <c r="N6" t="s">
-        <v>335</v>
+        <v>314</v>
       </c>
       <c r="O6" t="s">
-        <v>337</v>
+        <v>317</v>
       </c>
       <c r="P6" t="s">
-        <v>305</v>
+        <v>318</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>402</v>
       </c>
       <c r="R6">
-        <v>47.145499999999998</v>
+        <v>50.693460000000002</v>
       </c>
       <c r="S6">
-        <v>17.622399999999999</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>26</v>
+        <v>15.84652</v>
+      </c>
+      <c r="V6" t="s">
+        <v>405</v>
+      </c>
+      <c r="W6" t="s">
+        <v>30</v>
+      </c>
+      <c r="X6" s="2" t="s">
+        <v>400</v>
       </c>
     </row>
     <row r="7" spans="1:25" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>264</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>265</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>264</v>
+        <v>38</v>
       </c>
       <c r="D7" s="5">
-        <v>6011496</v>
+        <v>5755618</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>266</v>
+        <v>40</v>
       </c>
       <c r="F7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7">
+        <v>2015</v>
+      </c>
+      <c r="I7">
+        <v>2015</v>
+      </c>
+      <c r="J7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K7" t="s">
+        <v>43</v>
+      </c>
+      <c r="L7" t="s">
+        <v>20</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="N7" t="s">
+        <v>291</v>
+      </c>
+      <c r="O7" t="s">
+        <v>319</v>
+      </c>
+      <c r="P7" t="s">
+        <v>320</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>406</v>
+      </c>
+      <c r="R7">
+        <v>48.498627856338103</v>
+      </c>
+      <c r="S7">
+        <v>-89.227383734950806</v>
+      </c>
+      <c r="T7" t="s">
+        <v>415</v>
+      </c>
+      <c r="U7" t="s">
+        <v>414</v>
+      </c>
+      <c r="V7" t="s">
+        <v>321</v>
+      </c>
+      <c r="W7" t="s">
+        <v>412</v>
+      </c>
+      <c r="X7" s="2" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" ht="17" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="5">
+        <v>5755619</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H8">
+        <v>2015</v>
+      </c>
+      <c r="I8">
+        <v>2015</v>
+      </c>
+      <c r="J8" t="s">
+        <v>42</v>
+      </c>
+      <c r="K8" t="s">
+        <v>43</v>
+      </c>
+      <c r="L8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="N8" t="s">
+        <v>291</v>
+      </c>
+      <c r="O8" t="s">
+        <v>319</v>
+      </c>
+      <c r="P8" t="s">
+        <v>320</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>406</v>
+      </c>
+      <c r="R8">
+        <v>48.498627856338103</v>
+      </c>
+      <c r="S8">
+        <v>-89.227383734950806</v>
+      </c>
+      <c r="T8" t="s">
+        <v>415</v>
+      </c>
+      <c r="U8" t="s">
+        <v>414</v>
+      </c>
+      <c r="V8" t="s">
+        <v>321</v>
+      </c>
+      <c r="W8" t="s">
+        <v>413</v>
+      </c>
+      <c r="X8" s="2" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" ht="34" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" s="5">
+        <v>5755620</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" t="s">
         <v>51</v>
       </c>
-      <c r="G7" t="s">
-        <v>267</v>
-      </c>
-      <c r="H7">
-        <v>2011</v>
-      </c>
-      <c r="I7" s="1">
-        <v>40577</v>
-      </c>
-      <c r="J7" t="s">
-        <v>117</v>
-      </c>
-      <c r="K7" t="s">
-        <v>43</v>
-      </c>
-      <c r="L7" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="M7" s="32" t="s">
-        <v>427</v>
-      </c>
-      <c r="N7" t="s">
-        <v>268</v>
-      </c>
-      <c r="O7" t="s">
-        <v>305</v>
-      </c>
-      <c r="P7" t="s">
-        <v>305</v>
-      </c>
-      <c r="R7">
-        <v>50.45</v>
-      </c>
-      <c r="S7">
-        <v>30.5</v>
-      </c>
-      <c r="Y7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>269</v>
-      </c>
-      <c r="B8" t="s">
-        <v>270</v>
-      </c>
-      <c r="C8" t="s">
-        <v>269</v>
-      </c>
-      <c r="D8" s="5">
-        <v>6011497</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="F8" t="s">
-        <v>51</v>
-      </c>
-      <c r="G8" t="s">
-        <v>272</v>
-      </c>
-      <c r="H8">
-        <v>2009</v>
-      </c>
-      <c r="I8" s="1">
-        <v>39884</v>
-      </c>
-      <c r="J8" t="s">
-        <v>117</v>
-      </c>
-      <c r="K8" t="s">
-        <v>43</v>
-      </c>
-      <c r="L8" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="M8" s="32" t="s">
-        <v>427</v>
-      </c>
-      <c r="N8" t="s">
-        <v>346</v>
-      </c>
-      <c r="O8" t="s">
-        <v>363</v>
-      </c>
-      <c r="P8" t="s">
-        <v>362</v>
-      </c>
-      <c r="R8">
-        <v>45.1</v>
-      </c>
-      <c r="S8">
-        <v>0.7</v>
-      </c>
-      <c r="Y8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:25" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="5">
-        <v>3545531</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" t="s">
-        <v>16</v>
-      </c>
       <c r="G9" t="s">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="H9">
-        <v>2016</v>
+        <v>2013</v>
       </c>
       <c r="I9">
-        <v>2016</v>
+        <v>2013</v>
       </c>
       <c r="J9" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="K9" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="L9" t="s">
         <v>20</v>
@@ -7487,329 +7546,290 @@
         <v>305</v>
       </c>
       <c r="N9" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="O9" t="s">
-        <v>302</v>
+        <v>322</v>
       </c>
       <c r="P9" t="s">
-        <v>309</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>406</v>
-      </c>
-      <c r="R9" s="8">
-        <v>43.0274</v>
-      </c>
-      <c r="S9" s="8">
-        <v>-90.092200000000005</v>
-      </c>
-      <c r="X9" s="6" t="s">
-        <v>408</v>
-      </c>
-      <c r="Y9" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="10" spans="1:25" ht="51" x14ac:dyDescent="0.2">
+        <v>305</v>
+      </c>
+      <c r="R9">
+        <v>45.003125911591702</v>
+      </c>
+      <c r="S9">
+        <v>-63.830206168139703</v>
+      </c>
+      <c r="V9" t="s">
+        <v>307</v>
+      </c>
+      <c r="X9" s="2" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>54</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="D10" s="5">
-        <v>3411506</v>
+        <v>5755621</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="F10" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G10" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="H10">
-        <v>2010</v>
+        <v>2013</v>
       </c>
       <c r="I10">
-        <v>2010</v>
+        <v>2013</v>
       </c>
       <c r="J10" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="K10" t="s">
-        <v>19</v>
-      </c>
-      <c r="L10" s="10" t="s">
-        <v>25</v>
+        <v>43</v>
+      </c>
+      <c r="L10" t="s">
+        <v>20</v>
       </c>
       <c r="M10" s="7" t="s">
         <v>305</v>
       </c>
       <c r="N10" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="O10" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="P10" t="s">
-        <v>316</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>402</v>
+        <v>305</v>
       </c>
       <c r="R10">
-        <v>49.954439999999998</v>
+        <v>45.003125911591702</v>
       </c>
       <c r="S10">
-        <v>14.175829999999999</v>
+        <v>-63.830206168139703</v>
       </c>
       <c r="V10" t="s">
-        <v>403</v>
-      </c>
-      <c r="W10" t="s">
-        <v>401</v>
-      </c>
-      <c r="X10" s="2" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="11" spans="1:25" ht="51" x14ac:dyDescent="0.2">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="C11" t="s">
-        <v>27</v>
+        <v>57</v>
       </c>
       <c r="D11" s="5">
-        <v>3411507</v>
+        <v>5755622</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="F11" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G11" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H11">
-        <v>2010</v>
+        <v>2013</v>
       </c>
       <c r="I11">
-        <v>2010</v>
+        <v>2013</v>
       </c>
       <c r="J11" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="K11" t="s">
-        <v>19</v>
-      </c>
-      <c r="L11" s="10" t="s">
-        <v>25</v>
+        <v>43</v>
+      </c>
+      <c r="L11" t="s">
+        <v>20</v>
       </c>
       <c r="M11" s="7" t="s">
         <v>305</v>
       </c>
       <c r="N11" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="O11" t="s">
-        <v>315</v>
+        <v>295</v>
       </c>
       <c r="P11" t="s">
-        <v>316</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>402</v>
+        <v>305</v>
       </c>
       <c r="R11">
-        <v>49.954439999999998</v>
+        <v>46.011941999999998</v>
       </c>
       <c r="S11">
-        <v>14.175829999999999</v>
+        <v>-62.618592999999997</v>
       </c>
       <c r="V11" t="s">
-        <v>403</v>
-      </c>
-      <c r="W11" t="s">
-        <v>17</v>
-      </c>
-      <c r="X11" s="2" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="12" spans="1:25" ht="17" x14ac:dyDescent="0.2">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="C12" t="s">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="D12" s="5">
-        <v>3411508</v>
+        <v>5755623</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>33</v>
+        <v>63</v>
       </c>
       <c r="F12" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G12" t="s">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="H12">
-        <v>2011</v>
+        <v>2015</v>
       </c>
       <c r="I12">
-        <v>2011</v>
+        <v>2015</v>
       </c>
       <c r="J12" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="K12" t="s">
-        <v>19</v>
-      </c>
-      <c r="L12" s="10" t="s">
-        <v>25</v>
+        <v>43</v>
+      </c>
+      <c r="L12" t="s">
+        <v>20</v>
       </c>
       <c r="M12" s="7" t="s">
         <v>305</v>
       </c>
       <c r="N12" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="O12" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="P12" t="s">
-        <v>318</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>402</v>
+        <v>320</v>
       </c>
       <c r="R12">
-        <v>50.693460000000002</v>
+        <v>48.498627856338103</v>
       </c>
       <c r="S12">
-        <v>15.84652</v>
+        <v>-89.227383734950806</v>
       </c>
       <c r="V12" t="s">
-        <v>405</v>
-      </c>
-      <c r="W12" t="s">
-        <v>24</v>
-      </c>
-      <c r="X12" s="6" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="13" spans="1:25" ht="17" x14ac:dyDescent="0.2">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="D13" s="5">
-        <v>3411509</v>
+        <v>5755624</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="F13" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G13" t="s">
-        <v>13</v>
+        <v>68</v>
       </c>
       <c r="H13">
-        <v>2011</v>
+        <v>2015</v>
       </c>
       <c r="I13">
-        <v>2011</v>
+        <v>2015</v>
       </c>
       <c r="J13" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="K13" t="s">
-        <v>19</v>
-      </c>
-      <c r="L13" s="10" t="s">
-        <v>25</v>
+        <v>43</v>
+      </c>
+      <c r="L13" t="s">
+        <v>20</v>
       </c>
       <c r="M13" s="7" t="s">
         <v>305</v>
       </c>
       <c r="N13" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="O13" t="s">
-        <v>317</v>
+        <v>292</v>
       </c>
       <c r="P13" t="s">
-        <v>318</v>
-      </c>
-      <c r="Q13" t="s">
-        <v>402</v>
+        <v>293</v>
       </c>
       <c r="R13">
-        <v>50.693460000000002</v>
+        <v>45.913153999999999</v>
       </c>
       <c r="S13">
-        <v>15.84652</v>
+        <v>-64.671137999999999</v>
       </c>
       <c r="V13" t="s">
-        <v>405</v>
-      </c>
-      <c r="W13" t="s">
-        <v>30</v>
-      </c>
-      <c r="X13" s="2" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="14" spans="1:25" ht="17" x14ac:dyDescent="0.2">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="C14" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="D14" s="5">
-        <v>5755618</v>
+        <v>5755625</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="F14" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G14" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="H14">
-        <v>2015</v>
+        <v>2012</v>
       </c>
       <c r="I14">
-        <v>2015</v>
+        <v>2012</v>
       </c>
       <c r="J14" t="s">
         <v>42</v>
@@ -7827,63 +7847,48 @@
         <v>291</v>
       </c>
       <c r="O14" t="s">
-        <v>319</v>
+        <v>292</v>
       </c>
       <c r="P14" t="s">
-        <v>320</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>406</v>
+        <v>308</v>
       </c>
       <c r="R14">
-        <v>48.498627856338103</v>
+        <v>45.8172</v>
       </c>
       <c r="S14">
-        <v>-89.227383734950806</v>
-      </c>
-      <c r="T14" t="s">
-        <v>415</v>
-      </c>
-      <c r="U14" t="s">
-        <v>414</v>
+        <v>-65.610500000000002</v>
       </c>
       <c r="V14" t="s">
-        <v>321</v>
-      </c>
-      <c r="W14" t="s">
-        <v>412</v>
-      </c>
-      <c r="X14" s="2" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25" ht="17" x14ac:dyDescent="0.2">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>44</v>
+        <v>73</v>
       </c>
       <c r="B15" t="s">
-        <v>45</v>
+        <v>74</v>
       </c>
       <c r="C15" t="s">
-        <v>44</v>
+        <v>73</v>
       </c>
       <c r="D15" s="5">
-        <v>5755619</v>
+        <v>5755626</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="F15" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G15" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="H15">
-        <v>2015</v>
+        <v>2013</v>
       </c>
       <c r="I15">
-        <v>2015</v>
+        <v>2013</v>
       </c>
       <c r="J15" t="s">
         <v>42</v>
@@ -7901,63 +7906,48 @@
         <v>291</v>
       </c>
       <c r="O15" t="s">
-        <v>319</v>
+        <v>292</v>
       </c>
       <c r="P15" t="s">
-        <v>320</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>406</v>
+        <v>308</v>
       </c>
       <c r="R15">
-        <v>48.498627856338103</v>
+        <v>45.8172</v>
       </c>
       <c r="S15">
-        <v>-89.227383734950806</v>
-      </c>
-      <c r="T15" t="s">
-        <v>415</v>
-      </c>
-      <c r="U15" t="s">
-        <v>414</v>
+        <v>-65.610500000000002</v>
       </c>
       <c r="V15" t="s">
-        <v>321</v>
-      </c>
-      <c r="W15" t="s">
-        <v>413</v>
-      </c>
-      <c r="X15" s="2" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="16" spans="1:25" ht="34" x14ac:dyDescent="0.2">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>48</v>
+        <v>77</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>78</v>
       </c>
       <c r="C16" t="s">
-        <v>48</v>
+        <v>77</v>
       </c>
       <c r="D16" s="5">
-        <v>5755620</v>
+        <v>5755627</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="F16" t="s">
         <v>51</v>
       </c>
       <c r="G16" t="s">
-        <v>52</v>
+        <v>80</v>
       </c>
       <c r="H16">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="I16">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="J16" t="s">
         <v>42</v>
@@ -7975,51 +7965,48 @@
         <v>291</v>
       </c>
       <c r="O16" t="s">
-        <v>322</v>
+        <v>292</v>
       </c>
       <c r="P16" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="R16">
-        <v>45.003125911591702</v>
+        <v>45.913153999999999</v>
       </c>
       <c r="S16">
-        <v>-63.830206168139703</v>
+        <v>-64.671137999999999</v>
       </c>
       <c r="V16" t="s">
         <v>307</v>
       </c>
-      <c r="X16" s="2" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="B17" t="s">
-        <v>54</v>
+        <v>82</v>
       </c>
       <c r="C17" t="s">
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="D17" s="5">
-        <v>5755621</v>
+        <v>5755628</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>55</v>
+        <v>83</v>
       </c>
       <c r="F17" t="s">
         <v>51</v>
       </c>
       <c r="G17" t="s">
-        <v>56</v>
+        <v>84</v>
       </c>
       <c r="H17">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="I17">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="J17" t="s">
         <v>42</v>
@@ -8037,48 +8024,48 @@
         <v>291</v>
       </c>
       <c r="O17" t="s">
-        <v>322</v>
+        <v>292</v>
       </c>
       <c r="P17" t="s">
-        <v>305</v>
+        <v>294</v>
       </c>
       <c r="R17">
-        <v>45.003125911591702</v>
+        <v>45.615960000000001</v>
       </c>
       <c r="S17">
-        <v>-63.830206168139703</v>
+        <v>-65.439909999999998</v>
       </c>
       <c r="V17" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>85</v>
       </c>
       <c r="B18" t="s">
-        <v>58</v>
+        <v>86</v>
       </c>
       <c r="C18" t="s">
-        <v>57</v>
+        <v>85</v>
       </c>
       <c r="D18" s="5">
-        <v>5755622</v>
+        <v>5755629</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>59</v>
+        <v>87</v>
       </c>
       <c r="F18" t="s">
         <v>51</v>
       </c>
       <c r="G18" t="s">
-        <v>60</v>
+        <v>88</v>
       </c>
       <c r="H18">
-        <v>2013</v>
+        <v>2009</v>
       </c>
       <c r="I18">
-        <v>2013</v>
+        <v>2009</v>
       </c>
       <c r="J18" t="s">
         <v>42</v>
@@ -8086,58 +8073,58 @@
       <c r="K18" t="s">
         <v>43</v>
       </c>
-      <c r="L18" t="s">
-        <v>20</v>
+      <c r="L18" s="10" t="s">
+        <v>25</v>
       </c>
       <c r="M18" s="7" t="s">
         <v>305</v>
       </c>
       <c r="N18" t="s">
-        <v>291</v>
+        <v>323</v>
       </c>
       <c r="O18" t="s">
-        <v>295</v>
+        <v>324</v>
       </c>
       <c r="P18" t="s">
         <v>305</v>
       </c>
       <c r="R18">
-        <v>46.011941999999998</v>
+        <v>50.788476564399403</v>
       </c>
       <c r="S18">
-        <v>-62.618592999999997</v>
+        <v>10.740499703414899</v>
       </c>
       <c r="V18" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="19" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="B19" t="s">
-        <v>62</v>
+        <v>90</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="D19" s="5">
-        <v>5755623</v>
+        <v>5755630</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>63</v>
+        <v>91</v>
       </c>
       <c r="F19" t="s">
         <v>51</v>
       </c>
       <c r="G19" t="s">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="H19">
-        <v>2015</v>
+        <v>2013</v>
       </c>
       <c r="I19">
-        <v>2015</v>
+        <v>2013</v>
       </c>
       <c r="J19" t="s">
         <v>42</v>
@@ -8155,48 +8142,48 @@
         <v>291</v>
       </c>
       <c r="O19" t="s">
-        <v>319</v>
+        <v>292</v>
       </c>
       <c r="P19" t="s">
-        <v>320</v>
+        <v>297</v>
       </c>
       <c r="R19">
-        <v>48.498627856338103</v>
+        <v>45.93694</v>
       </c>
       <c r="S19">
-        <v>-89.227383734950806</v>
+        <v>-64.476939999999999</v>
       </c>
       <c r="V19" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="20" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="B20" t="s">
-        <v>66</v>
+        <v>94</v>
       </c>
       <c r="C20" t="s">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="D20" s="5">
-        <v>5755624</v>
+        <v>5755631</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="F20" t="s">
         <v>51</v>
       </c>
       <c r="G20" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="H20">
-        <v>2015</v>
+        <v>2013</v>
       </c>
       <c r="I20">
-        <v>2015</v>
+        <v>2013</v>
       </c>
       <c r="J20" t="s">
         <v>42</v>
@@ -8217,45 +8204,45 @@
         <v>292</v>
       </c>
       <c r="P20" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="R20">
-        <v>45.913153999999999</v>
+        <v>45.615960000000001</v>
       </c>
       <c r="S20">
-        <v>-64.671137999999999</v>
+        <v>-65.439909999999998</v>
       </c>
       <c r="V20" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="C21" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="D21" s="5">
-        <v>5755625</v>
+        <v>5755632</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>71</v>
+        <v>99</v>
       </c>
       <c r="F21" t="s">
         <v>51</v>
       </c>
       <c r="G21" t="s">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="H21">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="I21">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="J21" t="s">
         <v>42</v>
@@ -8276,39 +8263,39 @@
         <v>292</v>
       </c>
       <c r="P21" t="s">
-        <v>308</v>
+        <v>294</v>
       </c>
       <c r="R21">
-        <v>45.8172</v>
+        <v>45.615960000000001</v>
       </c>
       <c r="S21">
-        <v>-65.610500000000002</v>
+        <v>-65.439909999999998</v>
       </c>
       <c r="V21" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>73</v>
+        <v>101</v>
       </c>
       <c r="B22" t="s">
-        <v>74</v>
+        <v>102</v>
       </c>
       <c r="C22" t="s">
-        <v>73</v>
+        <v>101</v>
       </c>
       <c r="D22" s="5">
-        <v>5755626</v>
+        <v>5755633</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>75</v>
+        <v>103</v>
       </c>
       <c r="F22" t="s">
         <v>51</v>
       </c>
       <c r="G22" t="s">
-        <v>76</v>
+        <v>104</v>
       </c>
       <c r="H22">
         <v>2013</v>
@@ -8347,33 +8334,33 @@
         <v>307</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>77</v>
+        <v>105</v>
       </c>
       <c r="B23" t="s">
-        <v>78</v>
+        <v>106</v>
       </c>
       <c r="C23" t="s">
-        <v>77</v>
+        <v>105</v>
       </c>
       <c r="D23" s="5">
-        <v>5755627</v>
+        <v>5755634</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="F23" t="s">
         <v>51</v>
       </c>
       <c r="G23" t="s">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="H23">
-        <v>2012</v>
+        <v>2008</v>
       </c>
       <c r="I23">
-        <v>2012</v>
+        <v>2008</v>
       </c>
       <c r="J23" t="s">
         <v>42</v>
@@ -8388,45 +8375,54 @@
         <v>305</v>
       </c>
       <c r="N23" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="O23" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="P23" t="s">
-        <v>293</v>
+        <v>300</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>406</v>
       </c>
       <c r="R23">
-        <v>45.913153999999999</v>
+        <v>41.844515371877698</v>
       </c>
       <c r="S23">
-        <v>-64.671137999999999</v>
+        <v>-74.098548155198898</v>
+      </c>
+      <c r="T23" t="s">
+        <v>415</v>
       </c>
       <c r="V23" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
+        <v>325</v>
+      </c>
+      <c r="W23" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="24" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
       <c r="B24" t="s">
-        <v>82</v>
+        <v>110</v>
       </c>
       <c r="C24" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
       <c r="D24" s="5">
-        <v>5755628</v>
+        <v>5757331</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>83</v>
+        <v>111</v>
       </c>
       <c r="F24" t="s">
         <v>51</v>
       </c>
       <c r="G24" t="s">
-        <v>84</v>
+        <v>112</v>
       </c>
       <c r="H24">
         <v>2012</v>
@@ -8453,107 +8449,104 @@
         <v>292</v>
       </c>
       <c r="P24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="R24">
-        <v>45.615960000000001</v>
+        <v>45.913153999999999</v>
       </c>
       <c r="S24">
-        <v>-65.439909999999998</v>
+        <v>-64.671137999999999</v>
       </c>
       <c r="V24" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>85</v>
+        <v>113</v>
       </c>
       <c r="B25" t="s">
-        <v>86</v>
+        <v>114</v>
       </c>
       <c r="C25" t="s">
-        <v>85</v>
+        <v>113</v>
       </c>
       <c r="D25" s="5">
-        <v>5755629</v>
+        <v>7191697</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>87</v>
+        <v>115</v>
       </c>
       <c r="F25" t="s">
         <v>51</v>
       </c>
       <c r="G25" t="s">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="H25">
-        <v>2009</v>
-      </c>
-      <c r="I25">
-        <v>2009</v>
+        <v>2012</v>
+      </c>
+      <c r="I25" s="1">
+        <v>41011</v>
       </c>
       <c r="J25" t="s">
-        <v>42</v>
+        <v>117</v>
       </c>
       <c r="K25" t="s">
         <v>43</v>
       </c>
-      <c r="L25" s="10" t="s">
-        <v>25</v>
+      <c r="L25" t="s">
+        <v>20</v>
       </c>
       <c r="M25" s="7" t="s">
         <v>305</v>
       </c>
       <c r="N25" t="s">
-        <v>323</v>
+        <v>291</v>
       </c>
       <c r="O25" t="s">
-        <v>324</v>
+        <v>292</v>
       </c>
       <c r="P25" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="R25">
-        <v>50.788476564399403</v>
+        <v>45.93694</v>
       </c>
       <c r="S25">
-        <v>10.740499703414899</v>
-      </c>
-      <c r="V25" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.2">
+        <v>-64.476939999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
       <c r="B26" t="s">
-        <v>90</v>
+        <v>119</v>
       </c>
       <c r="C26" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
       <c r="D26" s="5">
-        <v>5755630</v>
+        <v>7191698</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>91</v>
+        <v>120</v>
       </c>
       <c r="F26" t="s">
         <v>51</v>
       </c>
       <c r="G26" t="s">
-        <v>92</v>
+        <v>121</v>
       </c>
       <c r="H26">
-        <v>2013</v>
-      </c>
-      <c r="I26">
-        <v>2013</v>
+        <v>2012</v>
+      </c>
+      <c r="I26" s="1">
+        <v>41013</v>
       </c>
       <c r="J26" t="s">
-        <v>42</v>
+        <v>117</v>
       </c>
       <c r="K26" t="s">
         <v>43</v>
@@ -8568,51 +8561,48 @@
         <v>291</v>
       </c>
       <c r="O26" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="P26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="R26">
-        <v>45.93694</v>
+        <v>46.011941999999998</v>
       </c>
       <c r="S26">
-        <v>-64.476939999999999</v>
-      </c>
-      <c r="V26" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.2">
+        <v>-62.618592999999997</v>
+      </c>
+    </row>
+    <row r="27" spans="1:25" ht="51" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>93</v>
+        <v>122</v>
       </c>
       <c r="B27" t="s">
-        <v>94</v>
+        <v>123</v>
       </c>
       <c r="C27" t="s">
-        <v>93</v>
+        <v>122</v>
       </c>
       <c r="D27" s="5">
-        <v>5755631</v>
+        <v>1952982</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>95</v>
+        <v>124</v>
       </c>
       <c r="F27" t="s">
         <v>51</v>
       </c>
       <c r="G27" t="s">
-        <v>96</v>
+        <v>125</v>
       </c>
       <c r="H27">
-        <v>2013</v>
+        <v>2008</v>
       </c>
       <c r="I27">
-        <v>2013</v>
+        <v>2008</v>
       </c>
       <c r="J27" t="s">
-        <v>42</v>
+        <v>117</v>
       </c>
       <c r="K27" t="s">
         <v>43</v>
@@ -8620,61 +8610,76 @@
       <c r="L27" t="s">
         <v>20</v>
       </c>
-      <c r="M27" s="7" t="s">
-        <v>305</v>
+      <c r="M27" t="s">
+        <v>427</v>
       </c>
       <c r="N27" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="O27" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="P27" t="s">
-        <v>294</v>
+        <v>328</v>
       </c>
       <c r="R27">
-        <v>45.615960000000001</v>
+        <v>41.844515371877698</v>
       </c>
       <c r="S27">
-        <v>-65.439909999999998</v>
+        <v>-74.098548155198898</v>
+      </c>
+      <c r="T27" t="s">
+        <v>379</v>
+      </c>
+      <c r="U27" t="s">
+        <v>380</v>
       </c>
       <c r="V27" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.2">
+        <v>378</v>
+      </c>
+      <c r="W27" t="s">
+        <v>384</v>
+      </c>
+      <c r="X27" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="Y27" s="2" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="28" spans="1:25" ht="34" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>97</v>
+        <v>154</v>
       </c>
       <c r="B28" t="s">
-        <v>98</v>
+        <v>155</v>
       </c>
       <c r="C28" t="s">
-        <v>97</v>
+        <v>154</v>
       </c>
       <c r="D28" s="5">
-        <v>5755632</v>
+        <v>29259</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>99</v>
+        <v>156</v>
       </c>
       <c r="F28" t="s">
         <v>51</v>
       </c>
       <c r="G28" t="s">
-        <v>100</v>
+        <v>157</v>
       </c>
       <c r="H28">
-        <v>2013</v>
-      </c>
-      <c r="I28">
-        <v>2013</v>
+        <v>2009</v>
+      </c>
+      <c r="I28" s="1">
+        <v>40073</v>
       </c>
       <c r="J28" t="s">
-        <v>42</v>
+        <v>158</v>
       </c>
       <c r="K28" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="L28" t="s">
         <v>20</v>
@@ -8683,57 +8688,72 @@
         <v>305</v>
       </c>
       <c r="N28" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="O28" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="P28" t="s">
-        <v>294</v>
+        <v>328</v>
       </c>
       <c r="R28">
-        <v>45.615960000000001</v>
+        <v>41.844515371877698</v>
       </c>
       <c r="S28">
-        <v>-65.439909999999998</v>
+        <v>-74.098548155198898</v>
+      </c>
+      <c r="T28" t="s">
+        <v>381</v>
+      </c>
+      <c r="U28" t="s">
+        <v>382</v>
       </c>
       <c r="V28" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.2">
+        <v>330</v>
+      </c>
+      <c r="W28" t="s">
+        <v>384</v>
+      </c>
+      <c r="X28" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="Y28" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="29" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>101</v>
+        <v>154</v>
       </c>
       <c r="B29" t="s">
-        <v>102</v>
+        <v>159</v>
       </c>
       <c r="C29" t="s">
-        <v>101</v>
+        <v>154</v>
       </c>
       <c r="D29" s="5">
-        <v>5755633</v>
+        <v>29260</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>103</v>
+        <v>160</v>
       </c>
       <c r="F29" t="s">
         <v>51</v>
       </c>
       <c r="G29" t="s">
-        <v>104</v>
+        <v>161</v>
       </c>
       <c r="H29">
-        <v>2013</v>
-      </c>
-      <c r="I29">
-        <v>2013</v>
+        <v>2009</v>
+      </c>
+      <c r="I29" s="1">
+        <v>40073</v>
       </c>
       <c r="J29" t="s">
-        <v>42</v>
+        <v>158</v>
       </c>
       <c r="K29" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="L29" t="s">
         <v>20</v>
@@ -8742,54 +8762,69 @@
         <v>305</v>
       </c>
       <c r="N29" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="O29" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="P29" t="s">
-        <v>308</v>
+        <v>328</v>
       </c>
       <c r="R29">
-        <v>45.8172</v>
+        <v>41.844515371877698</v>
       </c>
       <c r="S29">
-        <v>-65.610500000000002</v>
+        <v>-74.098548155198898</v>
+      </c>
+      <c r="T29" t="s">
+        <v>381</v>
+      </c>
+      <c r="U29" t="s">
+        <v>382</v>
       </c>
       <c r="V29" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.2">
+        <v>330</v>
+      </c>
+      <c r="W29" t="s">
+        <v>384</v>
+      </c>
+      <c r="X29" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="Y29" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="30" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>105</v>
+        <v>154</v>
       </c>
       <c r="B30" t="s">
-        <v>106</v>
+        <v>162</v>
       </c>
       <c r="C30" t="s">
-        <v>105</v>
+        <v>154</v>
       </c>
       <c r="D30" s="5">
-        <v>5755634</v>
+        <v>31784</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>107</v>
+        <v>163</v>
       </c>
       <c r="F30" t="s">
         <v>51</v>
       </c>
       <c r="G30" t="s">
-        <v>108</v>
+        <v>164</v>
       </c>
       <c r="H30">
-        <v>2008</v>
-      </c>
-      <c r="I30">
-        <v>2008</v>
+        <v>2009</v>
+      </c>
+      <c r="I30" s="1">
+        <v>40073</v>
       </c>
       <c r="J30" t="s">
-        <v>42</v>
+        <v>158</v>
       </c>
       <c r="K30" t="s">
         <v>43</v>
@@ -8807,10 +8842,7 @@
         <v>299</v>
       </c>
       <c r="P30" t="s">
-        <v>300</v>
-      </c>
-      <c r="Q30" t="s">
-        <v>406</v>
+        <v>328</v>
       </c>
       <c r="R30">
         <v>41.844515371877698</v>
@@ -8819,45 +8851,54 @@
         <v>-74.098548155198898</v>
       </c>
       <c r="T30" t="s">
-        <v>415</v>
+        <v>381</v>
+      </c>
+      <c r="U30" t="s">
+        <v>382</v>
       </c>
       <c r="V30" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="W30" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.2">
+        <v>384</v>
+      </c>
+      <c r="X30" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="Y30" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="31" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>109</v>
+        <v>154</v>
       </c>
       <c r="B31" t="s">
-        <v>110</v>
+        <v>165</v>
       </c>
       <c r="C31" t="s">
-        <v>109</v>
+        <v>154</v>
       </c>
       <c r="D31" s="5">
-        <v>5757331</v>
+        <v>107675</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>111</v>
+        <v>166</v>
       </c>
       <c r="F31" t="s">
         <v>51</v>
       </c>
       <c r="G31" t="s">
-        <v>112</v>
+        <v>167</v>
       </c>
       <c r="H31">
-        <v>2012</v>
-      </c>
-      <c r="I31">
-        <v>2012</v>
+        <v>2009</v>
+      </c>
+      <c r="I31" s="1">
+        <v>40073</v>
       </c>
       <c r="J31" t="s">
-        <v>42</v>
+        <v>158</v>
       </c>
       <c r="K31" t="s">
         <v>43</v>
@@ -8869,169 +8910,190 @@
         <v>305</v>
       </c>
       <c r="N31" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="O31" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="P31" t="s">
-        <v>293</v>
+        <v>328</v>
       </c>
       <c r="R31">
-        <v>45.913153999999999</v>
+        <v>41.844515371877698</v>
       </c>
       <c r="S31">
-        <v>-64.671137999999999</v>
+        <v>-74.098548155198898</v>
+      </c>
+      <c r="T31" t="s">
+        <v>381</v>
+      </c>
+      <c r="U31" t="s">
+        <v>382</v>
       </c>
       <c r="V31" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.2">
+        <v>330</v>
+      </c>
+      <c r="W31" t="s">
+        <v>384</v>
+      </c>
+      <c r="X31" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="Y31" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="32" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>113</v>
+        <v>168</v>
       </c>
       <c r="B32" t="s">
-        <v>114</v>
+        <v>169</v>
       </c>
       <c r="C32" t="s">
-        <v>113</v>
+        <v>168</v>
       </c>
       <c r="D32" s="5">
-        <v>7191697</v>
+        <v>6011467</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>115</v>
+        <v>170</v>
       </c>
       <c r="F32" t="s">
         <v>51</v>
       </c>
       <c r="G32" t="s">
-        <v>116</v>
+        <v>171</v>
       </c>
       <c r="H32">
-        <v>2012</v>
+        <v>2009</v>
       </c>
       <c r="I32" s="1">
-        <v>41011</v>
+        <v>39879</v>
       </c>
       <c r="J32" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="K32" t="s">
         <v>43</v>
       </c>
-      <c r="L32" t="s">
-        <v>20</v>
-      </c>
-      <c r="M32" s="7" t="s">
+      <c r="L32" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="M32" t="s">
+        <v>427</v>
+      </c>
+      <c r="N32" t="s">
+        <v>323</v>
+      </c>
+      <c r="O32" t="s">
+        <v>324</v>
+      </c>
+      <c r="P32" t="s">
         <v>305</v>
       </c>
-      <c r="N32" t="s">
-        <v>291</v>
-      </c>
-      <c r="O32" t="s">
-        <v>292</v>
-      </c>
-      <c r="P32" t="s">
-        <v>297</v>
-      </c>
       <c r="R32">
-        <v>45.93694</v>
+        <v>50.788476564399403</v>
       </c>
       <c r="S32">
-        <v>-64.476939999999999</v>
+        <v>10.740499703414899</v>
+      </c>
+      <c r="Y32" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="33" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
       <c r="B33" t="s">
-        <v>119</v>
+        <v>172</v>
       </c>
       <c r="C33" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
       <c r="D33" s="5">
-        <v>7191698</v>
+        <v>6011468</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>120</v>
+        <v>173</v>
       </c>
       <c r="F33" t="s">
         <v>51</v>
       </c>
       <c r="G33" t="s">
-        <v>121</v>
+        <v>174</v>
       </c>
       <c r="H33">
-        <v>2012</v>
+        <v>2009</v>
       </c>
       <c r="I33" s="1">
-        <v>41013</v>
+        <v>39904</v>
       </c>
       <c r="J33" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="K33" t="s">
         <v>43</v>
       </c>
-      <c r="L33" t="s">
-        <v>20</v>
-      </c>
-      <c r="M33" s="7" t="s">
+      <c r="L33" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="M33" t="s">
+        <v>427</v>
+      </c>
+      <c r="N33" t="s">
+        <v>336</v>
+      </c>
+      <c r="O33" t="s">
+        <v>338</v>
+      </c>
+      <c r="P33" t="s">
         <v>305</v>
       </c>
-      <c r="N33" t="s">
-        <v>291</v>
-      </c>
-      <c r="O33" t="s">
-        <v>295</v>
-      </c>
-      <c r="P33" t="s">
-        <v>296</v>
-      </c>
       <c r="R33">
-        <v>46.011941999999998</v>
+        <v>47.083329999999997</v>
       </c>
       <c r="S33">
-        <v>-62.618592999999997</v>
-      </c>
-    </row>
-    <row r="34" spans="1:25" ht="34" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="Y33" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>154</v>
+        <v>174</v>
       </c>
       <c r="B34" t="s">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="C34" t="s">
-        <v>154</v>
+        <v>174</v>
       </c>
       <c r="D34" s="5">
-        <v>29259</v>
+        <v>6011469</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>156</v>
+        <v>176</v>
       </c>
       <c r="F34" t="s">
         <v>51</v>
       </c>
       <c r="G34" t="s">
-        <v>157</v>
+        <v>177</v>
       </c>
       <c r="H34">
         <v>2009</v>
       </c>
       <c r="I34" s="1">
-        <v>40073</v>
+        <v>39897</v>
       </c>
       <c r="J34" t="s">
-        <v>158</v>
+        <v>130</v>
       </c>
       <c r="K34" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="L34" t="s">
         <v>20</v>
@@ -9043,69 +9105,51 @@
         <v>298</v>
       </c>
       <c r="O34" t="s">
-        <v>299</v>
+        <v>339</v>
       </c>
       <c r="P34" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="R34">
-        <v>41.844515371877698</v>
+        <v>40.888610999999997</v>
       </c>
       <c r="S34">
-        <v>-74.098548155198898</v>
-      </c>
-      <c r="T34" t="s">
-        <v>381</v>
-      </c>
-      <c r="U34" t="s">
-        <v>382</v>
-      </c>
-      <c r="V34" t="s">
-        <v>330</v>
-      </c>
-      <c r="W34" t="s">
-        <v>384</v>
-      </c>
-      <c r="X34" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="Y34" s="2" t="s">
-        <v>327</v>
+        <v>-77.386111</v>
       </c>
     </row>
     <row r="35" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="B35" t="s">
-        <v>159</v>
+        <v>178</v>
       </c>
       <c r="C35" t="s">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="D35" s="5">
-        <v>29260</v>
+        <v>6011470</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>160</v>
+        <v>179</v>
       </c>
       <c r="F35" t="s">
         <v>51</v>
       </c>
       <c r="G35" t="s">
-        <v>161</v>
+        <v>180</v>
       </c>
       <c r="H35">
         <v>2009</v>
       </c>
       <c r="I35" s="1">
-        <v>40073</v>
+        <v>39990</v>
       </c>
       <c r="J35" t="s">
-        <v>158</v>
+        <v>130</v>
       </c>
       <c r="K35" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="L35" t="s">
         <v>20</v>
@@ -9117,66 +9161,48 @@
         <v>298</v>
       </c>
       <c r="O35" t="s">
-        <v>299</v>
+        <v>341</v>
       </c>
       <c r="P35" t="s">
-        <v>328</v>
+        <v>342</v>
       </c>
       <c r="R35">
-        <v>41.844515371877698</v>
+        <v>40.877385651285401</v>
       </c>
       <c r="S35">
-        <v>-74.098548155198898</v>
-      </c>
-      <c r="T35" t="s">
-        <v>381</v>
-      </c>
-      <c r="U35" t="s">
-        <v>382</v>
-      </c>
-      <c r="V35" t="s">
-        <v>330</v>
-      </c>
-      <c r="W35" t="s">
-        <v>384</v>
-      </c>
-      <c r="X35" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="Y35" t="s">
-        <v>331</v>
+        <v>-74.968855407371393</v>
       </c>
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>154</v>
+        <v>180</v>
       </c>
       <c r="B36" t="s">
-        <v>162</v>
+        <v>181</v>
       </c>
       <c r="C36" t="s">
-        <v>154</v>
+        <v>180</v>
       </c>
       <c r="D36" s="5">
-        <v>31784</v>
+        <v>6011471</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
       <c r="F36" t="s">
         <v>51</v>
       </c>
       <c r="G36" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="H36">
         <v>2009</v>
       </c>
       <c r="I36" s="1">
-        <v>40073</v>
+        <v>39843</v>
       </c>
       <c r="J36" t="s">
-        <v>158</v>
+        <v>130</v>
       </c>
       <c r="K36" t="s">
         <v>43</v>
@@ -9191,66 +9217,48 @@
         <v>298</v>
       </c>
       <c r="O36" t="s">
-        <v>299</v>
+        <v>343</v>
       </c>
       <c r="P36" t="s">
-        <v>328</v>
+        <v>344</v>
       </c>
       <c r="R36">
-        <v>41.844515371877698</v>
+        <v>38.664935999999997</v>
       </c>
       <c r="S36">
-        <v>-74.098548155198898</v>
-      </c>
-      <c r="T36" t="s">
-        <v>381</v>
-      </c>
-      <c r="U36" t="s">
-        <v>382</v>
-      </c>
-      <c r="V36" t="s">
-        <v>330</v>
-      </c>
-      <c r="W36" t="s">
-        <v>384</v>
-      </c>
-      <c r="X36" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="Y36" t="s">
-        <v>331</v>
+        <v>-79.430160999999998</v>
       </c>
     </row>
     <row r="37" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>154</v>
+        <v>183</v>
       </c>
       <c r="B37" t="s">
-        <v>165</v>
+        <v>184</v>
       </c>
       <c r="C37" t="s">
-        <v>154</v>
+        <v>183</v>
       </c>
       <c r="D37" s="5">
-        <v>107675</v>
+        <v>6011472</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>166</v>
+        <v>185</v>
       </c>
       <c r="F37" t="s">
         <v>51</v>
       </c>
       <c r="G37" t="s">
-        <v>167</v>
+        <v>186</v>
       </c>
       <c r="H37">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="I37" s="1">
-        <v>40073</v>
+        <v>40248</v>
       </c>
       <c r="J37" t="s">
-        <v>158</v>
+        <v>130</v>
       </c>
       <c r="K37" t="s">
         <v>43</v>
@@ -9262,66 +9270,48 @@
         <v>305</v>
       </c>
       <c r="N37" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="O37" t="s">
-        <v>299</v>
+        <v>319</v>
       </c>
       <c r="P37" t="s">
-        <v>328</v>
+        <v>345</v>
       </c>
       <c r="R37">
-        <v>41.844515371877698</v>
+        <v>48.174337000000001</v>
       </c>
       <c r="S37">
-        <v>-74.098548155198898</v>
-      </c>
-      <c r="T37" t="s">
-        <v>381</v>
-      </c>
-      <c r="U37" t="s">
-        <v>382</v>
-      </c>
-      <c r="V37" t="s">
-        <v>330</v>
-      </c>
-      <c r="W37" t="s">
-        <v>384</v>
-      </c>
-      <c r="X37" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="Y37" t="s">
-        <v>331</v>
+        <v>-80.100126000000003</v>
       </c>
     </row>
     <row r="38" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="B38" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="C38" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="D38" s="5">
-        <v>6011469</v>
+        <v>6011473</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="F38" t="s">
         <v>51</v>
       </c>
       <c r="G38" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="H38">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="I38" s="1">
-        <v>39897</v>
+        <v>40242</v>
       </c>
       <c r="J38" t="s">
         <v>130</v>
@@ -9339,48 +9329,48 @@
         <v>298</v>
       </c>
       <c r="O38" t="s">
-        <v>339</v>
+        <v>354</v>
       </c>
       <c r="P38" t="s">
-        <v>340</v>
+        <v>366</v>
       </c>
       <c r="R38">
-        <v>40.888610999999997</v>
+        <v>36.555458999999999</v>
       </c>
       <c r="S38">
-        <v>-77.386111</v>
+        <v>-87.304068999999998</v>
       </c>
     </row>
     <row r="39" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="B39" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="C39" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="D39" s="5">
-        <v>6011470</v>
+        <v>6011474</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="F39" t="s">
         <v>51</v>
       </c>
       <c r="G39" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="H39">
-        <v>2009</v>
+        <v>2008</v>
       </c>
       <c r="I39" s="1">
-        <v>39990</v>
+        <v>39525</v>
       </c>
       <c r="J39" t="s">
-        <v>130</v>
+        <v>193</v>
       </c>
       <c r="K39" t="s">
         <v>43</v>
@@ -9395,45 +9385,45 @@
         <v>298</v>
       </c>
       <c r="O39" t="s">
-        <v>341</v>
+        <v>304</v>
       </c>
       <c r="P39" t="s">
-        <v>342</v>
+        <v>360</v>
       </c>
       <c r="R39">
-        <v>40.877385651285401</v>
+        <v>42.871989999999997</v>
       </c>
       <c r="S39">
-        <v>-74.968855407371393</v>
+        <v>-73.226607000000001</v>
       </c>
     </row>
     <row r="40" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="B40" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="C40" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="D40" s="5">
-        <v>6011471</v>
+        <v>6011475</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="F40" t="s">
         <v>51</v>
       </c>
       <c r="G40" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="H40">
         <v>2009</v>
       </c>
       <c r="I40" s="1">
-        <v>39843</v>
+        <v>39840</v>
       </c>
       <c r="J40" t="s">
         <v>130</v>
@@ -9451,45 +9441,45 @@
         <v>298</v>
       </c>
       <c r="O40" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="P40" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="R40">
-        <v>38.664935999999997</v>
+        <v>41.745700999999997</v>
       </c>
       <c r="S40">
-        <v>-79.430160999999998</v>
+        <v>-73.158473999999998</v>
       </c>
     </row>
     <row r="41" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="B41" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="C41" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="D41" s="5">
-        <v>6011472</v>
+        <v>6011476</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="F41" t="s">
         <v>51</v>
       </c>
       <c r="G41" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="H41">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="I41" s="1">
-        <v>40248</v>
+        <v>39875</v>
       </c>
       <c r="J41" t="s">
         <v>130</v>
@@ -9504,48 +9494,48 @@
         <v>305</v>
       </c>
       <c r="N41" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="O41" t="s">
-        <v>319</v>
+        <v>351</v>
       </c>
       <c r="P41" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="R41">
-        <v>48.174337000000001</v>
+        <v>37.322156999999997</v>
       </c>
       <c r="S41">
-        <v>-80.100126000000003</v>
+        <v>-80.756189000000006</v>
       </c>
     </row>
     <row r="42" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="B42" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="C42" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="D42" s="5">
-        <v>6011473</v>
+        <v>6011477</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="F42" t="s">
         <v>51</v>
       </c>
       <c r="G42" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="H42">
-        <v>2010</v>
+        <v>2008</v>
       </c>
       <c r="I42" s="1">
-        <v>40242</v>
+        <v>39528</v>
       </c>
       <c r="J42" t="s">
         <v>130</v>
@@ -9563,51 +9553,51 @@
         <v>298</v>
       </c>
       <c r="O42" t="s">
-        <v>354</v>
+        <v>348</v>
       </c>
       <c r="P42" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="R42">
-        <v>36.555458999999999</v>
+        <v>42.592351000000001</v>
       </c>
       <c r="S42">
-        <v>-87.304068999999998</v>
-      </c>
-    </row>
-    <row r="43" spans="1:25" x14ac:dyDescent="0.2">
+        <v>-73.226241999999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:25" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>189</v>
+        <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="C43" t="s">
-        <v>189</v>
+        <v>41</v>
       </c>
       <c r="D43" s="5">
-        <v>6011474</v>
+        <v>3545532</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="F43" t="s">
         <v>51</v>
       </c>
       <c r="G43" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="H43">
-        <v>2008</v>
-      </c>
-      <c r="I43" s="1">
-        <v>39525</v>
+        <v>2015</v>
+      </c>
+      <c r="I43">
+        <v>2015</v>
       </c>
       <c r="J43" t="s">
-        <v>193</v>
+        <v>18</v>
       </c>
       <c r="K43" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="L43" t="s">
         <v>20</v>
@@ -9619,51 +9609,60 @@
         <v>298</v>
       </c>
       <c r="O43" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="P43" t="s">
-        <v>360</v>
+        <v>311</v>
+      </c>
+      <c r="Q43" t="s">
+        <v>407</v>
       </c>
       <c r="R43">
-        <v>42.871989999999997</v>
+        <v>34.574328000000001</v>
       </c>
       <c r="S43">
-        <v>-73.226607000000001</v>
-      </c>
-    </row>
-    <row r="44" spans="1:25" x14ac:dyDescent="0.2">
+        <v>-86.220834999999994</v>
+      </c>
+      <c r="X43" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="Y43" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="44" spans="1:25" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>192</v>
+        <v>47</v>
       </c>
       <c r="B44" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="C44" t="s">
-        <v>192</v>
+        <v>47</v>
       </c>
       <c r="D44" s="5">
-        <v>6011475</v>
+        <v>3545533</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="F44" t="s">
         <v>51</v>
       </c>
       <c r="G44" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="H44">
-        <v>2009</v>
-      </c>
-      <c r="I44" s="1">
-        <v>39840</v>
+        <v>2016</v>
+      </c>
+      <c r="I44">
+        <v>2016</v>
       </c>
       <c r="J44" t="s">
-        <v>130</v>
+        <v>18</v>
       </c>
       <c r="K44" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="L44" t="s">
         <v>20</v>
@@ -9675,45 +9674,54 @@
         <v>298</v>
       </c>
       <c r="O44" t="s">
-        <v>349</v>
+        <v>312</v>
       </c>
       <c r="P44" t="s">
-        <v>350</v>
+        <v>313</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>406</v>
       </c>
       <c r="R44">
-        <v>41.745700999999997</v>
+        <v>47.550894599999999</v>
       </c>
       <c r="S44">
-        <v>-73.158473999999998</v>
+        <v>-121.53941880000001</v>
+      </c>
+      <c r="X44" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="Y44" t="s">
+        <v>411</v>
       </c>
     </row>
     <row r="45" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="B45" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="C45" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="D45" s="5">
-        <v>6011476</v>
+        <v>6011465</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="F45" t="s">
         <v>51</v>
       </c>
       <c r="G45" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="H45">
         <v>2009</v>
       </c>
       <c r="I45" s="1">
-        <v>39875</v>
+        <v>39901</v>
       </c>
       <c r="J45" t="s">
         <v>130</v>
@@ -9721,55 +9729,58 @@
       <c r="K45" t="s">
         <v>43</v>
       </c>
-      <c r="L45" t="s">
-        <v>20</v>
-      </c>
-      <c r="M45" s="7" t="s">
+      <c r="L45" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="M45" t="s">
+        <v>427</v>
+      </c>
+      <c r="N45" t="s">
+        <v>335</v>
+      </c>
+      <c r="O45" t="s">
+        <v>337</v>
+      </c>
+      <c r="P45" t="s">
         <v>305</v>
       </c>
-      <c r="N45" t="s">
-        <v>298</v>
-      </c>
-      <c r="O45" t="s">
-        <v>351</v>
-      </c>
-      <c r="P45" t="s">
-        <v>352</v>
-      </c>
       <c r="R45">
-        <v>37.322156999999997</v>
+        <v>47.145499999999998</v>
       </c>
       <c r="S45">
-        <v>-80.756189000000006</v>
+        <v>17.622399999999999</v>
+      </c>
+      <c r="Y45" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="46" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B46" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="C46" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D46" s="5">
-        <v>6011477</v>
+        <v>6011478</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="F46" t="s">
         <v>51</v>
       </c>
       <c r="G46" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="H46">
         <v>2008</v>
       </c>
       <c r="I46" s="1">
-        <v>39528</v>
+        <v>39539</v>
       </c>
       <c r="J46" t="s">
         <v>130</v>
@@ -9787,51 +9798,51 @@
         <v>298</v>
       </c>
       <c r="O46" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="P46" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="R46">
-        <v>42.592351000000001</v>
+        <v>41.745700999999997</v>
       </c>
       <c r="S46">
-        <v>-73.226241999999999</v>
-      </c>
-    </row>
-    <row r="47" spans="1:25" ht="17" x14ac:dyDescent="0.2">
+        <v>-73.158473999999998</v>
+      </c>
+    </row>
+    <row r="47" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>41</v>
+        <v>205</v>
       </c>
       <c r="B47" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="C47" t="s">
-        <v>41</v>
+        <v>205</v>
       </c>
       <c r="D47" s="5">
-        <v>3545532</v>
+        <v>6011479</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="F47" t="s">
         <v>51</v>
       </c>
       <c r="G47" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="H47">
-        <v>2015</v>
-      </c>
-      <c r="I47">
-        <v>2015</v>
+        <v>2010</v>
+      </c>
+      <c r="I47" s="1">
+        <v>40217</v>
       </c>
       <c r="J47" t="s">
-        <v>18</v>
+        <v>130</v>
       </c>
       <c r="K47" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="L47" t="s">
         <v>20</v>
@@ -9843,60 +9854,51 @@
         <v>298</v>
       </c>
       <c r="O47" t="s">
-        <v>310</v>
+        <v>354</v>
       </c>
       <c r="P47" t="s">
-        <v>311</v>
-      </c>
-      <c r="Q47" t="s">
-        <v>407</v>
+        <v>365</v>
       </c>
       <c r="R47">
-        <v>34.574328000000001</v>
+        <v>36.509321</v>
       </c>
       <c r="S47">
-        <v>-86.220834999999994</v>
-      </c>
-      <c r="X47" s="6" t="s">
-        <v>408</v>
-      </c>
-      <c r="Y47" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="48" spans="1:25" ht="17" x14ac:dyDescent="0.2">
+        <v>-82.328933000000006</v>
+      </c>
+    </row>
+    <row r="48" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>47</v>
+        <v>208</v>
       </c>
       <c r="B48" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="C48" t="s">
-        <v>47</v>
+        <v>208</v>
       </c>
       <c r="D48" s="5">
-        <v>3545533</v>
+        <v>6011480</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="F48" t="s">
         <v>51</v>
       </c>
       <c r="G48" t="s">
-        <v>208</v>
+        <v>129</v>
       </c>
       <c r="H48">
-        <v>2016</v>
-      </c>
-      <c r="I48">
-        <v>2016</v>
+        <v>2010</v>
+      </c>
+      <c r="I48" s="1">
+        <v>40242</v>
       </c>
       <c r="J48" t="s">
-        <v>18</v>
+        <v>130</v>
       </c>
       <c r="K48" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="L48" t="s">
         <v>20</v>
@@ -9908,57 +9910,51 @@
         <v>298</v>
       </c>
       <c r="O48" t="s">
-        <v>312</v>
+        <v>355</v>
       </c>
       <c r="P48" t="s">
-        <v>313</v>
-      </c>
-      <c r="Q48" t="s">
-        <v>406</v>
+        <v>367</v>
       </c>
       <c r="R48">
-        <v>47.550894599999999</v>
+        <v>39.69717</v>
       </c>
       <c r="S48">
-        <v>-121.53941880000001</v>
-      </c>
-      <c r="X48" s="6" t="s">
-        <v>408</v>
-      </c>
-      <c r="Y48" t="s">
-        <v>411</v>
+        <v>-78.820670000000007</v>
+      </c>
+      <c r="Y48" s="9" t="s">
+        <v>417</v>
       </c>
     </row>
     <row r="49" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="B49" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="C49" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="D49" s="5">
-        <v>6011478</v>
+        <v>6011481</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="F49" t="s">
         <v>51</v>
       </c>
       <c r="G49" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="H49">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="I49" s="1">
-        <v>39539</v>
+        <v>39882</v>
       </c>
       <c r="J49" t="s">
-        <v>130</v>
+        <v>193</v>
       </c>
       <c r="K49" t="s">
         <v>43</v>
@@ -9973,45 +9969,45 @@
         <v>298</v>
       </c>
       <c r="O49" t="s">
-        <v>349</v>
+        <v>299</v>
       </c>
       <c r="P49" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="R49">
-        <v>41.745700999999997</v>
+        <v>41.949971359391597</v>
       </c>
       <c r="S49">
-        <v>-73.158473999999998</v>
+        <v>-74.288489118822994</v>
       </c>
     </row>
     <row r="50" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>205</v>
+        <v>134</v>
       </c>
       <c r="B50" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="C50" t="s">
-        <v>205</v>
+        <v>134</v>
       </c>
       <c r="D50" s="5">
-        <v>6011479</v>
+        <v>6011482</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="F50" t="s">
         <v>51</v>
       </c>
       <c r="G50" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="H50">
         <v>2010</v>
       </c>
       <c r="I50" s="1">
-        <v>40217</v>
+        <v>40205</v>
       </c>
       <c r="J50" t="s">
         <v>130</v>
@@ -10029,45 +10025,45 @@
         <v>298</v>
       </c>
       <c r="O50" t="s">
-        <v>354</v>
+        <v>304</v>
       </c>
       <c r="P50" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="R50">
-        <v>36.509321</v>
+        <v>43.451169999999998</v>
       </c>
       <c r="S50">
-        <v>-82.328933000000006</v>
+        <v>-72.942554999999999</v>
       </c>
     </row>
     <row r="51" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>208</v>
+        <v>138</v>
       </c>
       <c r="B51" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="C51" t="s">
-        <v>208</v>
+        <v>138</v>
       </c>
       <c r="D51" s="5">
-        <v>6011480</v>
+        <v>6011483</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="F51" t="s">
         <v>51</v>
       </c>
       <c r="G51" t="s">
-        <v>129</v>
+        <v>229</v>
       </c>
       <c r="H51">
         <v>2010</v>
       </c>
       <c r="I51" s="1">
-        <v>40242</v>
+        <v>40252</v>
       </c>
       <c r="J51" t="s">
         <v>130</v>
@@ -10082,54 +10078,51 @@
         <v>305</v>
       </c>
       <c r="N51" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="O51" t="s">
-        <v>355</v>
+        <v>319</v>
       </c>
       <c r="P51" t="s">
-        <v>367</v>
+        <v>305</v>
       </c>
       <c r="R51">
-        <v>39.69717</v>
+        <v>48.174337000000001</v>
       </c>
       <c r="S51">
-        <v>-78.820670000000007</v>
-      </c>
-      <c r="Y51" s="9" t="s">
-        <v>417</v>
+        <v>-80.100126000000003</v>
       </c>
     </row>
     <row r="52" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>212</v>
+        <v>142</v>
       </c>
       <c r="B52" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="C52" t="s">
-        <v>212</v>
+        <v>142</v>
       </c>
       <c r="D52" s="5">
-        <v>6011481</v>
+        <v>6011484</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="F52" t="s">
-        <v>51</v>
+        <v>232</v>
       </c>
       <c r="G52" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="H52">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="I52" s="1">
-        <v>39882</v>
+        <v>40275</v>
       </c>
       <c r="J52" t="s">
-        <v>193</v>
+        <v>130</v>
       </c>
       <c r="K52" t="s">
         <v>43</v>
@@ -10144,157 +10137,157 @@
         <v>298</v>
       </c>
       <c r="O52" t="s">
-        <v>299</v>
+        <v>354</v>
       </c>
       <c r="P52" t="s">
-        <v>353</v>
+        <v>368</v>
       </c>
       <c r="R52">
-        <v>41.949971359391597</v>
+        <v>36.465316000000001</v>
       </c>
       <c r="S52">
-        <v>-74.288489118822994</v>
+        <v>-84.971273999999994</v>
       </c>
     </row>
     <row r="53" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="B53" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="C53" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="D53" s="5">
-        <v>6011482</v>
+        <v>6011486</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="F53" t="s">
-        <v>51</v>
+        <v>232</v>
       </c>
       <c r="G53" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="H53">
-        <v>2010</v>
-      </c>
-      <c r="I53" s="1">
-        <v>40205</v>
+        <v>2016</v>
+      </c>
+      <c r="I53">
+        <v>2016</v>
       </c>
       <c r="J53" t="s">
-        <v>130</v>
+        <v>42</v>
       </c>
       <c r="K53" t="s">
         <v>43</v>
       </c>
-      <c r="L53" t="s">
-        <v>20</v>
-      </c>
-      <c r="M53" s="7" t="s">
+      <c r="L53" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="M53" t="s">
+        <v>428</v>
+      </c>
+      <c r="N53" t="s">
+        <v>237</v>
+      </c>
+      <c r="O53" t="s">
         <v>305</v>
       </c>
-      <c r="N53" t="s">
-        <v>298</v>
-      </c>
-      <c r="O53" t="s">
-        <v>304</v>
-      </c>
       <c r="P53" t="s">
-        <v>364</v>
+        <v>237</v>
       </c>
       <c r="R53">
-        <v>43.451169999999998</v>
+        <v>46.823079999999997</v>
       </c>
       <c r="S53">
-        <v>-72.942554999999999</v>
+        <v>102.503703</v>
       </c>
     </row>
     <row r="54" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="B54" t="s">
-        <v>227</v>
+        <v>238</v>
       </c>
       <c r="C54" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="D54" s="5">
-        <v>6011483</v>
+        <v>6011487</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="F54" t="s">
-        <v>51</v>
+        <v>232</v>
       </c>
       <c r="G54" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="H54">
-        <v>2010</v>
-      </c>
-      <c r="I54" s="1">
-        <v>40252</v>
+        <v>2016</v>
+      </c>
+      <c r="I54">
+        <v>2016</v>
       </c>
       <c r="J54" t="s">
-        <v>130</v>
+        <v>42</v>
       </c>
       <c r="K54" t="s">
         <v>43</v>
       </c>
-      <c r="L54" t="s">
-        <v>20</v>
+      <c r="L54" s="10" t="s">
+        <v>236</v>
       </c>
       <c r="M54" s="7" t="s">
         <v>305</v>
       </c>
       <c r="N54" t="s">
-        <v>291</v>
+        <v>237</v>
       </c>
       <c r="O54" t="s">
-        <v>319</v>
+        <v>305</v>
       </c>
       <c r="P54" t="s">
-        <v>305</v>
+        <v>237</v>
       </c>
       <c r="R54">
-        <v>48.174337000000001</v>
+        <v>46.823079999999997</v>
       </c>
       <c r="S54">
-        <v>-80.100126000000003</v>
+        <v>102.503703</v>
       </c>
     </row>
     <row r="55" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="B55" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
       <c r="C55" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="D55" s="5">
-        <v>6011484</v>
+        <v>6011488</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>231</v>
+        <v>242</v>
       </c>
       <c r="F55" t="s">
         <v>232</v>
       </c>
       <c r="G55" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="H55">
-        <v>2010</v>
+        <v>2012</v>
       </c>
       <c r="I55" s="1">
-        <v>40275</v>
+        <v>41011</v>
       </c>
       <c r="J55" t="s">
         <v>130</v>
@@ -10309,104 +10302,104 @@
         <v>305</v>
       </c>
       <c r="N55" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="O55" t="s">
-        <v>354</v>
+        <v>292</v>
       </c>
       <c r="P55" t="s">
-        <v>368</v>
+        <v>297</v>
       </c>
       <c r="R55">
-        <v>36.465316000000001</v>
+        <v>45.93694</v>
       </c>
       <c r="S55">
-        <v>-84.971273999999994</v>
+        <v>-64.476939999999999</v>
       </c>
     </row>
     <row r="56" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="B56" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="C56" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="D56" s="5">
-        <v>6011487</v>
+        <v>6011489</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="F56" t="s">
         <v>232</v>
       </c>
       <c r="G56" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="H56">
-        <v>2016</v>
-      </c>
-      <c r="I56">
-        <v>2016</v>
+        <v>2012</v>
+      </c>
+      <c r="I56" s="1">
+        <v>40987</v>
       </c>
       <c r="J56" t="s">
-        <v>42</v>
+        <v>117</v>
       </c>
       <c r="K56" t="s">
         <v>43</v>
       </c>
-      <c r="L56" s="10" t="s">
-        <v>236</v>
+      <c r="L56" t="s">
+        <v>20</v>
       </c>
       <c r="M56" s="7" t="s">
         <v>305</v>
       </c>
       <c r="N56" t="s">
-        <v>237</v>
+        <v>298</v>
       </c>
       <c r="O56" t="s">
-        <v>305</v>
+        <v>359</v>
       </c>
       <c r="P56" t="s">
-        <v>237</v>
+        <v>374</v>
       </c>
       <c r="R56">
-        <v>46.823079999999997</v>
+        <v>39.048609999999996</v>
       </c>
       <c r="S56">
-        <v>102.503703</v>
+        <v>-90.88167</v>
       </c>
     </row>
     <row r="57" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>157</v>
+        <v>246</v>
       </c>
       <c r="B57" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="C57" t="s">
-        <v>157</v>
+        <v>246</v>
       </c>
       <c r="D57" s="5">
-        <v>6011488</v>
+        <v>6011490</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="F57" t="s">
         <v>232</v>
       </c>
       <c r="G57" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="H57">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="I57" s="1">
-        <v>41011</v>
+        <v>40590</v>
       </c>
       <c r="J57" t="s">
         <v>130</v>
@@ -10421,51 +10414,51 @@
         <v>305</v>
       </c>
       <c r="N57" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="O57" t="s">
-        <v>292</v>
+        <v>351</v>
       </c>
       <c r="P57" t="s">
-        <v>297</v>
+        <v>371</v>
       </c>
       <c r="R57">
-        <v>45.93694</v>
+        <v>36.968234063873403</v>
       </c>
       <c r="S57">
-        <v>-64.476939999999999</v>
+        <v>-82.639469435652799</v>
       </c>
     </row>
     <row r="58" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B58" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="C58" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D58" s="5">
-        <v>6011489</v>
+        <v>6011491</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="F58" t="s">
         <v>232</v>
       </c>
       <c r="G58" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="H58">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="I58" s="1">
-        <v>40987</v>
+        <v>40583</v>
       </c>
       <c r="J58" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="K58" t="s">
         <v>43</v>
@@ -10480,45 +10473,45 @@
         <v>298</v>
       </c>
       <c r="O58" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="P58" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="R58">
-        <v>39.048609999999996</v>
+        <v>36.555458999999999</v>
       </c>
       <c r="S58">
-        <v>-90.88167</v>
+        <v>-87.304068999999998</v>
       </c>
     </row>
     <row r="59" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B59" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C59" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D59" s="5">
-        <v>6011490</v>
+        <v>6011492</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F59" t="s">
         <v>232</v>
       </c>
       <c r="G59" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="H59">
         <v>2011</v>
       </c>
       <c r="I59" s="1">
-        <v>40590</v>
+        <v>40572</v>
       </c>
       <c r="J59" t="s">
         <v>130</v>
@@ -10536,48 +10529,48 @@
         <v>298</v>
       </c>
       <c r="O59" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="P59" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="R59">
-        <v>36.968234063873403</v>
+        <v>38.229909999999997</v>
       </c>
       <c r="S59">
-        <v>-82.639469435652799</v>
+        <v>-86.294910000000002</v>
       </c>
     </row>
     <row r="60" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>164</v>
+        <v>254</v>
       </c>
       <c r="B60" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="C60" t="s">
-        <v>164</v>
+        <v>254</v>
       </c>
       <c r="D60" s="5">
-        <v>6011491</v>
+        <v>6011493</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="F60" t="s">
         <v>232</v>
       </c>
       <c r="G60" t="s">
-        <v>240</v>
+        <v>257</v>
       </c>
       <c r="H60">
         <v>2011</v>
       </c>
       <c r="I60" s="1">
-        <v>40583</v>
+        <v>40566</v>
       </c>
       <c r="J60" t="s">
-        <v>130</v>
+        <v>193</v>
       </c>
       <c r="K60" t="s">
         <v>43</v>
@@ -10592,48 +10585,48 @@
         <v>298</v>
       </c>
       <c r="O60" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="P60" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="R60">
-        <v>36.555458999999999</v>
+        <v>38.702026438267701</v>
       </c>
       <c r="S60">
-        <v>-87.304068999999998</v>
+        <v>-86.233603821942907</v>
       </c>
     </row>
     <row r="61" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="B61" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="C61" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="D61" s="5">
-        <v>6011492</v>
+        <v>6011494</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="F61" t="s">
         <v>232</v>
       </c>
       <c r="G61" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
       <c r="H61">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="I61" s="1">
-        <v>40572</v>
+        <v>40969</v>
       </c>
       <c r="J61" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="K61" t="s">
         <v>43</v>
@@ -10648,48 +10641,48 @@
         <v>298</v>
       </c>
       <c r="O61" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="P61" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="R61">
-        <v>38.229909999999997</v>
+        <v>39.838700000000003</v>
       </c>
       <c r="S61">
-        <v>-86.294910000000002</v>
+        <v>-75.563800000000001</v>
       </c>
     </row>
     <row r="62" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>254</v>
+        <v>215</v>
       </c>
       <c r="B62" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="C62" t="s">
-        <v>254</v>
+        <v>215</v>
       </c>
       <c r="D62" s="5">
-        <v>6011493</v>
+        <v>6011495</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="F62" t="s">
-        <v>232</v>
+        <v>51</v>
       </c>
       <c r="G62" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="H62">
         <v>2011</v>
       </c>
       <c r="I62" s="1">
-        <v>40566</v>
+        <v>40889</v>
       </c>
       <c r="J62" t="s">
-        <v>193</v>
+        <v>117</v>
       </c>
       <c r="K62" t="s">
         <v>43</v>
@@ -10704,45 +10697,48 @@
         <v>298</v>
       </c>
       <c r="O62" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="P62" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="R62">
-        <v>38.702026438267701</v>
+        <v>44.349651999999999</v>
       </c>
       <c r="S62">
-        <v>-86.233603821942907</v>
+        <v>-68.211070000000007</v>
+      </c>
+      <c r="Y62" s="9" t="s">
+        <v>418</v>
       </c>
     </row>
     <row r="63" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="B63" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="C63" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="D63" s="5">
-        <v>6011494</v>
+        <v>6011496</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="F63" t="s">
-        <v>232</v>
+        <v>51</v>
       </c>
       <c r="G63" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="H63">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="I63" s="1">
-        <v>40969</v>
+        <v>40577</v>
       </c>
       <c r="J63" t="s">
         <v>117</v>
@@ -10750,55 +10746,58 @@
       <c r="K63" t="s">
         <v>43</v>
       </c>
-      <c r="L63" t="s">
-        <v>20</v>
-      </c>
-      <c r="M63" s="7" t="s">
+      <c r="L63" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="M63" t="s">
+        <v>427</v>
+      </c>
+      <c r="N63" t="s">
+        <v>268</v>
+      </c>
+      <c r="O63" t="s">
         <v>305</v>
       </c>
-      <c r="N63" t="s">
-        <v>298</v>
-      </c>
-      <c r="O63" t="s">
-        <v>358</v>
-      </c>
       <c r="P63" t="s">
-        <v>373</v>
+        <v>305</v>
       </c>
       <c r="R63">
-        <v>39.838700000000003</v>
+        <v>50.45</v>
       </c>
       <c r="S63">
-        <v>-75.563800000000001</v>
+        <v>30.5</v>
+      </c>
+      <c r="Y63" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="64" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>215</v>
+        <v>269</v>
       </c>
       <c r="B64" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C64" t="s">
-        <v>215</v>
+        <v>269</v>
       </c>
       <c r="D64" s="5">
-        <v>6011495</v>
+        <v>6011497</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="F64" t="s">
         <v>51</v>
       </c>
       <c r="G64" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="H64">
-        <v>2011</v>
+        <v>2009</v>
       </c>
       <c r="I64" s="1">
-        <v>40889</v>
+        <v>39884</v>
       </c>
       <c r="J64" t="s">
         <v>117</v>
@@ -10806,29 +10805,29 @@
       <c r="K64" t="s">
         <v>43</v>
       </c>
-      <c r="L64" t="s">
-        <v>20</v>
-      </c>
-      <c r="M64" s="7" t="s">
-        <v>305</v>
+      <c r="L64" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="M64" t="s">
+        <v>427</v>
       </c>
       <c r="N64" t="s">
-        <v>298</v>
+        <v>346</v>
       </c>
       <c r="O64" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="P64" t="s">
-        <v>372</v>
+        <v>362</v>
       </c>
       <c r="R64">
-        <v>44.349651999999999</v>
+        <v>45.1</v>
       </c>
       <c r="S64">
-        <v>-68.211070000000007</v>
-      </c>
-      <c r="Y64" s="9" t="s">
-        <v>418</v>
+        <v>0.7</v>
+      </c>
+      <c r="Y64" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="65" spans="1:19" x14ac:dyDescent="0.2">
@@ -11057,16 +11056,16 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="X34" r:id="rId1" xr:uid="{3DA3BF50-C718-4042-AB38-8735C412C066}"/>
+    <hyperlink ref="X28" r:id="rId1" xr:uid="{3DA3BF50-C718-4042-AB38-8735C412C066}"/>
     <hyperlink ref="X3:X5" r:id="rId2" display="https://www.broadinstitute.org/fungal-genome-initiative/geomyces-destructans-genome-project" xr:uid="{1AAC961A-6EDA-4148-9B4F-0CA1532C4848}"/>
-    <hyperlink ref="X3" r:id="rId3" xr:uid="{9413F2DF-9CF6-5A47-9263-53F94E6E38F0}"/>
+    <hyperlink ref="X27" r:id="rId3" xr:uid="{9413F2DF-9CF6-5A47-9263-53F94E6E38F0}"/>
     <hyperlink ref="X7:X13" r:id="rId4" display="https://doi.org/10.1038/s41467-017-02441-z" xr:uid="{10FFF060-2B2E-064B-83CE-CE5C13A4C475}"/>
-    <hyperlink ref="X12" r:id="rId5" xr:uid="{AA3197C4-28D6-7F45-809F-3D3F6942E815}"/>
-    <hyperlink ref="X9" r:id="rId6" xr:uid="{BD924FBD-C0DE-C744-B59B-8D2DA9D331DE}"/>
-    <hyperlink ref="X47" r:id="rId7" xr:uid="{90F9021C-5B1B-6240-BAA5-2E9F79A0155A}"/>
-    <hyperlink ref="X48" r:id="rId8" xr:uid="{2594ECE7-B238-6940-A003-2BD99A0CB6A2}"/>
-    <hyperlink ref="Y51" r:id="rId9" location="close --&gt; used to find  most clustered group of caves in the county" xr:uid="{92A2A68F-4C43-8149-AF16-4E3ECAC1437F}"/>
-    <hyperlink ref="Y64" r:id="rId10" xr:uid="{C7F50DBF-DBBD-8F40-84B6-E18DD5C9F49C}"/>
+    <hyperlink ref="X5" r:id="rId5" xr:uid="{AA3197C4-28D6-7F45-809F-3D3F6942E815}"/>
+    <hyperlink ref="X2" r:id="rId6" xr:uid="{BD924FBD-C0DE-C744-B59B-8D2DA9D331DE}"/>
+    <hyperlink ref="X43" r:id="rId7" xr:uid="{90F9021C-5B1B-6240-BAA5-2E9F79A0155A}"/>
+    <hyperlink ref="X44" r:id="rId8" xr:uid="{2594ECE7-B238-6940-A003-2BD99A0CB6A2}"/>
+    <hyperlink ref="Y48" r:id="rId9" location="close --&gt; used to find  most clustered group of caves in the county" xr:uid="{92A2A68F-4C43-8149-AF16-4E3ECAC1437F}"/>
+    <hyperlink ref="Y62" r:id="rId10" xr:uid="{C7F50DBF-DBBD-8F40-84B6-E18DD5C9F49C}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
new pca graphs for all n-amer samples
</commit_message>
<xml_diff>
--- a/data/01_pd-samples/26_01_15_pd_samples-edited.xlsx
+++ b/data/01_pd-samples/26_01_15_pd_samples-edited.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/caprinapugliese/Documents/03_school/Uconn/2024-26_Grad_School/Dagilis-lab/WNS-project/data/01_pd-samples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68EDBDDA-3160-7947-902B-79468568869F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A8F889-A087-A840-9517-8ED55CA43AD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6920" yWindow="2480" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{D99E271A-162C-F24C-8D0E-BBA6ED327C07}"/>
+    <workbookView xWindow="12860" yWindow="1620" windowWidth="24340" windowHeight="21100" activeTab="1" xr2:uid="{D99E271A-162C-F24C-8D0E-BBA6ED327C07}"/>
   </bookViews>
   <sheets>
     <sheet name="25_10-16_pd_samples-edited" sheetId="1" r:id="rId1"/>
@@ -1510,7 +1510,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1708,6 +1708,12 @@
         <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="12">
     <border>
@@ -1890,7 +1896,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1947,6 +1953,16 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="36" borderId="0" xfId="42" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -8647,299 +8663,299 @@
         <v>387</v>
       </c>
     </row>
-    <row r="28" spans="1:25" ht="34" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+    <row r="28" spans="1:25" s="32" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A28" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="32" t="s">
         <v>155</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="D28" s="5">
+      <c r="D28" s="33">
         <v>29259</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="34" t="s">
         <v>156</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F28" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G28" s="32" t="s">
         <v>157</v>
       </c>
-      <c r="H28">
+      <c r="H28" s="32">
         <v>2009</v>
       </c>
-      <c r="I28" s="1">
+      <c r="I28" s="35">
         <v>40073</v>
       </c>
-      <c r="J28" t="s">
+      <c r="J28" s="32" t="s">
         <v>158</v>
       </c>
-      <c r="K28" t="s">
+      <c r="K28" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="L28" t="s">
-        <v>20</v>
-      </c>
-      <c r="M28" s="7" t="s">
+      <c r="L28" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="M28" s="32" t="s">
         <v>305</v>
       </c>
-      <c r="N28" t="s">
+      <c r="N28" s="32" t="s">
         <v>298</v>
       </c>
-      <c r="O28" t="s">
+      <c r="O28" s="32" t="s">
         <v>299</v>
       </c>
-      <c r="P28" t="s">
+      <c r="P28" s="32" t="s">
         <v>328</v>
       </c>
-      <c r="R28">
+      <c r="R28" s="32">
         <v>41.844515371877698</v>
       </c>
-      <c r="S28">
+      <c r="S28" s="32">
         <v>-74.098548155198898</v>
       </c>
-      <c r="T28" t="s">
+      <c r="T28" s="32" t="s">
         <v>381</v>
       </c>
-      <c r="U28" t="s">
+      <c r="U28" s="32" t="s">
         <v>382</v>
       </c>
-      <c r="V28" t="s">
+      <c r="V28" s="32" t="s">
         <v>330</v>
       </c>
-      <c r="W28" t="s">
+      <c r="W28" s="32" t="s">
         <v>384</v>
       </c>
-      <c r="X28" s="3" t="s">
+      <c r="X28" s="36" t="s">
         <v>329</v>
       </c>
-      <c r="Y28" s="2" t="s">
+      <c r="Y28" s="37" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+    <row r="29" spans="1:25" s="32" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="32" t="s">
         <v>159</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="D29" s="5">
+      <c r="D29" s="33">
         <v>29260</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="34" t="s">
         <v>160</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="G29" t="s">
+      <c r="G29" s="32" t="s">
         <v>161</v>
       </c>
-      <c r="H29">
+      <c r="H29" s="32">
         <v>2009</v>
       </c>
-      <c r="I29" s="1">
+      <c r="I29" s="35">
         <v>40073</v>
       </c>
-      <c r="J29" t="s">
+      <c r="J29" s="32" t="s">
         <v>158</v>
       </c>
-      <c r="K29" t="s">
+      <c r="K29" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="L29" t="s">
-        <v>20</v>
-      </c>
-      <c r="M29" s="7" t="s">
+      <c r="L29" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="M29" s="32" t="s">
         <v>305</v>
       </c>
-      <c r="N29" t="s">
+      <c r="N29" s="32" t="s">
         <v>298</v>
       </c>
-      <c r="O29" t="s">
+      <c r="O29" s="32" t="s">
         <v>299</v>
       </c>
-      <c r="P29" t="s">
+      <c r="P29" s="32" t="s">
         <v>328</v>
       </c>
-      <c r="R29">
+      <c r="R29" s="32">
         <v>41.844515371877698</v>
       </c>
-      <c r="S29">
+      <c r="S29" s="32">
         <v>-74.098548155198898</v>
       </c>
-      <c r="T29" t="s">
+      <c r="T29" s="32" t="s">
         <v>381</v>
       </c>
-      <c r="U29" t="s">
+      <c r="U29" s="32" t="s">
         <v>382</v>
       </c>
-      <c r="V29" t="s">
+      <c r="V29" s="32" t="s">
         <v>330</v>
       </c>
-      <c r="W29" t="s">
+      <c r="W29" s="32" t="s">
         <v>384</v>
       </c>
-      <c r="X29" s="3" t="s">
+      <c r="X29" s="36" t="s">
         <v>329</v>
       </c>
-      <c r="Y29" t="s">
+      <c r="Y29" s="32" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+    <row r="30" spans="1:25" s="32" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="32" t="s">
         <v>162</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="D30" s="5">
+      <c r="D30" s="33">
         <v>31784</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="34" t="s">
         <v>163</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G30" s="32" t="s">
         <v>164</v>
       </c>
-      <c r="H30">
+      <c r="H30" s="32">
         <v>2009</v>
       </c>
-      <c r="I30" s="1">
+      <c r="I30" s="35">
         <v>40073</v>
       </c>
-      <c r="J30" t="s">
+      <c r="J30" s="32" t="s">
         <v>158</v>
       </c>
-      <c r="K30" t="s">
-        <v>43</v>
-      </c>
-      <c r="L30" t="s">
-        <v>20</v>
-      </c>
-      <c r="M30" s="7" t="s">
+      <c r="K30" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="L30" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="M30" s="32" t="s">
         <v>305</v>
       </c>
-      <c r="N30" t="s">
+      <c r="N30" s="32" t="s">
         <v>298</v>
       </c>
-      <c r="O30" t="s">
+      <c r="O30" s="32" t="s">
         <v>299</v>
       </c>
-      <c r="P30" t="s">
+      <c r="P30" s="32" t="s">
         <v>328</v>
       </c>
-      <c r="R30">
+      <c r="R30" s="32">
         <v>41.844515371877698</v>
       </c>
-      <c r="S30">
+      <c r="S30" s="32">
         <v>-74.098548155198898</v>
       </c>
-      <c r="T30" t="s">
+      <c r="T30" s="32" t="s">
         <v>381</v>
       </c>
-      <c r="U30" t="s">
+      <c r="U30" s="32" t="s">
         <v>382</v>
       </c>
-      <c r="V30" t="s">
+      <c r="V30" s="32" t="s">
         <v>330</v>
       </c>
-      <c r="W30" t="s">
+      <c r="W30" s="32" t="s">
         <v>384</v>
       </c>
-      <c r="X30" s="3" t="s">
+      <c r="X30" s="36" t="s">
         <v>329</v>
       </c>
-      <c r="Y30" t="s">
+      <c r="Y30" s="32" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+    <row r="31" spans="1:25" s="32" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="D31" s="5">
+      <c r="D31" s="33">
         <v>107675</v>
       </c>
-      <c r="E31" s="4" t="s">
+      <c r="E31" s="34" t="s">
         <v>166</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" s="32" t="s">
         <v>167</v>
       </c>
-      <c r="H31">
+      <c r="H31" s="32">
         <v>2009</v>
       </c>
-      <c r="I31" s="1">
+      <c r="I31" s="35">
         <v>40073</v>
       </c>
-      <c r="J31" t="s">
+      <c r="J31" s="32" t="s">
         <v>158</v>
       </c>
-      <c r="K31" t="s">
-        <v>43</v>
-      </c>
-      <c r="L31" t="s">
-        <v>20</v>
-      </c>
-      <c r="M31" s="7" t="s">
+      <c r="K31" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="L31" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="M31" s="32" t="s">
         <v>305</v>
       </c>
-      <c r="N31" t="s">
+      <c r="N31" s="32" t="s">
         <v>298</v>
       </c>
-      <c r="O31" t="s">
+      <c r="O31" s="32" t="s">
         <v>299</v>
       </c>
-      <c r="P31" t="s">
+      <c r="P31" s="32" t="s">
         <v>328</v>
       </c>
-      <c r="R31">
+      <c r="R31" s="32">
         <v>41.844515371877698</v>
       </c>
-      <c r="S31">
+      <c r="S31" s="32">
         <v>-74.098548155198898</v>
       </c>
-      <c r="T31" t="s">
+      <c r="T31" s="32" t="s">
         <v>381</v>
       </c>
-      <c r="U31" t="s">
+      <c r="U31" s="32" t="s">
         <v>382</v>
       </c>
-      <c r="V31" t="s">
+      <c r="V31" s="32" t="s">
         <v>330</v>
       </c>
-      <c r="W31" t="s">
+      <c r="W31" s="32" t="s">
         <v>384</v>
       </c>
-      <c r="X31" s="3" t="s">
+      <c r="X31" s="36" t="s">
         <v>329</v>
       </c>
-      <c r="Y31" t="s">
+      <c r="Y31" s="32" t="s">
         <v>331</v>
       </c>
     </row>

</xml_diff>

<commit_message>
made info for pcangsd for all samples
</commit_message>
<xml_diff>
--- a/data/01_pd-samples/26_01_15_pd_samples-edited.xlsx
+++ b/data/01_pd-samples/26_01_15_pd_samples-edited.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/caprinapugliese/Documents/03_school/Uconn/2024-26_Grad_School/Dagilis-lab/WNS-project/data/01_pd-samples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A8F889-A087-A840-9517-8ED55CA43AD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{037D8769-EDFA-084D-9744-ACC125216792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12860" yWindow="1620" windowWidth="24340" windowHeight="21100" activeTab="1" xr2:uid="{D99E271A-162C-F24C-8D0E-BBA6ED327C07}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="27800" windowHeight="17500" activeTab="6" xr2:uid="{D99E271A-162C-F24C-8D0E-BBA6ED327C07}"/>
   </bookViews>
   <sheets>
     <sheet name="25_10-16_pd_samples-edited" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="NoA_Pd_coords" sheetId="3" r:id="rId4"/>
     <sheet name="no washington" sheetId="5" r:id="rId5"/>
     <sheet name="no_washington_all_info" sheetId="8" r:id="rId6"/>
+    <sheet name="ALL_samples" sheetId="10" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3524" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4050" uniqueCount="434">
   <si>
     <t>sample_id</t>
   </si>
@@ -1326,6 +1327,21 @@
   </si>
   <si>
     <t>pd_2</t>
+  </si>
+  <si>
+    <t>group_names</t>
+  </si>
+  <si>
+    <t>P. species</t>
+  </si>
+  <si>
+    <t>lab_clone</t>
+  </si>
+  <si>
+    <t>group2</t>
+  </si>
+  <si>
+    <t>group1</t>
   </si>
 </sst>
 </file>
@@ -2162,6 +2178,23 @@
 </table>
 </file>
 
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{62A55085-0CF0-F740-A56A-7F09F21DA478}" name="Table15" displayName="Table15" ref="A1:H75" totalsRowShown="0">
+  <autoFilter ref="A1:H75" xr:uid="{90C14361-2949-B74A-BFF6-1CEFD0790204}"/>
+  <tableColumns count="8">
+    <tableColumn id="2" xr3:uid="{EF84A378-15D3-B54F-9A97-CBC8D4E6613E}" name="individuals"/>
+    <tableColumn id="24" xr3:uid="{E3A157CC-35C3-F345-A455-CB963B085872}" name="names"/>
+    <tableColumn id="18" xr3:uid="{CFCDA3AE-71A6-A040-8EED-8C168193D75E}" name="year"/>
+    <tableColumn id="9" xr3:uid="{E8ED157C-369B-A149-973D-EEC00B15CD00}" name="continent"/>
+    <tableColumn id="10" xr3:uid="{8DD2323C-C82D-0347-9C98-A81A2364584F}" name="country"/>
+    <tableColumn id="11" xr3:uid="{C059A186-EAB6-A74D-BB5A-40430B80B655}" name="state"/>
+    <tableColumn id="12" xr3:uid="{6C3CC1A4-61AD-F74F-920F-7068D49C5DB7}" name="location"/>
+    <tableColumn id="1" xr3:uid="{CC8B6DEC-F5E7-4E4B-81DD-DCFFA3CB9568}" name="group_names"/>
+  </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -18506,4 +18539,1977 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{386D9C2A-E883-BE41-A0C8-238F9C54EB0C}">
+  <dimension ref="A1:H75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="41.6640625" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" customWidth="1"/>
+    <col min="5" max="5" width="14.1640625" customWidth="1"/>
+    <col min="6" max="6" width="25.6640625" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>375</v>
+      </c>
+      <c r="B1" t="s">
+        <v>388</v>
+      </c>
+      <c r="C1" t="s">
+        <v>347</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
+        <v>290</v>
+      </c>
+      <c r="F1" t="s">
+        <v>289</v>
+      </c>
+      <c r="G1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2">
+        <v>2016</v>
+      </c>
+      <c r="D2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
+        <v>298</v>
+      </c>
+      <c r="F2" t="s">
+        <v>302</v>
+      </c>
+      <c r="G2" t="s">
+        <v>309</v>
+      </c>
+      <c r="H2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3">
+        <v>2010</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" t="s">
+        <v>314</v>
+      </c>
+      <c r="F3" t="s">
+        <v>315</v>
+      </c>
+      <c r="G3" t="s">
+        <v>316</v>
+      </c>
+      <c r="H3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4">
+        <v>2010</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" t="s">
+        <v>314</v>
+      </c>
+      <c r="F4" t="s">
+        <v>315</v>
+      </c>
+      <c r="G4" t="s">
+        <v>316</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5">
+        <v>2011</v>
+      </c>
+      <c r="D5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" t="s">
+        <v>314</v>
+      </c>
+      <c r="F5" t="s">
+        <v>317</v>
+      </c>
+      <c r="G5" t="s">
+        <v>318</v>
+      </c>
+      <c r="H5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6">
+        <v>2011</v>
+      </c>
+      <c r="D6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" t="s">
+        <v>314</v>
+      </c>
+      <c r="F6" t="s">
+        <v>317</v>
+      </c>
+      <c r="G6" t="s">
+        <v>318</v>
+      </c>
+      <c r="H6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7">
+        <v>2015</v>
+      </c>
+      <c r="D7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" t="s">
+        <v>291</v>
+      </c>
+      <c r="F7" t="s">
+        <v>319</v>
+      </c>
+      <c r="G7" t="s">
+        <v>320</v>
+      </c>
+      <c r="H7" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8">
+        <v>2015</v>
+      </c>
+      <c r="D8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" t="s">
+        <v>291</v>
+      </c>
+      <c r="F8" t="s">
+        <v>319</v>
+      </c>
+      <c r="G8" t="s">
+        <v>320</v>
+      </c>
+      <c r="H8" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9">
+        <v>2013</v>
+      </c>
+      <c r="D9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" t="s">
+        <v>291</v>
+      </c>
+      <c r="F9" t="s">
+        <v>322</v>
+      </c>
+      <c r="G9" t="s">
+        <v>305</v>
+      </c>
+      <c r="H9" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10">
+        <v>2013</v>
+      </c>
+      <c r="D10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" t="s">
+        <v>291</v>
+      </c>
+      <c r="F10" t="s">
+        <v>322</v>
+      </c>
+      <c r="G10" t="s">
+        <v>305</v>
+      </c>
+      <c r="H10" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11">
+        <v>2013</v>
+      </c>
+      <c r="D11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" t="s">
+        <v>291</v>
+      </c>
+      <c r="F11" t="s">
+        <v>295</v>
+      </c>
+      <c r="G11" t="s">
+        <v>305</v>
+      </c>
+      <c r="H11" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12">
+        <v>2015</v>
+      </c>
+      <c r="D12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" t="s">
+        <v>291</v>
+      </c>
+      <c r="F12" t="s">
+        <v>319</v>
+      </c>
+      <c r="G12" t="s">
+        <v>320</v>
+      </c>
+      <c r="H12" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13">
+        <v>2015</v>
+      </c>
+      <c r="D13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" t="s">
+        <v>291</v>
+      </c>
+      <c r="F13" t="s">
+        <v>292</v>
+      </c>
+      <c r="G13" t="s">
+        <v>293</v>
+      </c>
+      <c r="H13" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14">
+        <v>2012</v>
+      </c>
+      <c r="D14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" t="s">
+        <v>291</v>
+      </c>
+      <c r="F14" t="s">
+        <v>292</v>
+      </c>
+      <c r="G14" t="s">
+        <v>308</v>
+      </c>
+      <c r="H14" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15">
+        <v>2013</v>
+      </c>
+      <c r="D15" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" t="s">
+        <v>291</v>
+      </c>
+      <c r="F15" t="s">
+        <v>292</v>
+      </c>
+      <c r="G15" t="s">
+        <v>308</v>
+      </c>
+      <c r="H15" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16">
+        <v>2012</v>
+      </c>
+      <c r="D16" t="s">
+        <v>20</v>
+      </c>
+      <c r="E16" t="s">
+        <v>291</v>
+      </c>
+      <c r="F16" t="s">
+        <v>292</v>
+      </c>
+      <c r="G16" t="s">
+        <v>293</v>
+      </c>
+      <c r="H16" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" t="s">
+        <v>81</v>
+      </c>
+      <c r="C17">
+        <v>2012</v>
+      </c>
+      <c r="D17" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" t="s">
+        <v>291</v>
+      </c>
+      <c r="F17" t="s">
+        <v>292</v>
+      </c>
+      <c r="G17" t="s">
+        <v>294</v>
+      </c>
+      <c r="H17" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>86</v>
+      </c>
+      <c r="B18" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18">
+        <v>2009</v>
+      </c>
+      <c r="D18" t="s">
+        <v>25</v>
+      </c>
+      <c r="E18" t="s">
+        <v>323</v>
+      </c>
+      <c r="F18" t="s">
+        <v>324</v>
+      </c>
+      <c r="G18" t="s">
+        <v>305</v>
+      </c>
+      <c r="H18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>90</v>
+      </c>
+      <c r="B19" t="s">
+        <v>89</v>
+      </c>
+      <c r="C19">
+        <v>2013</v>
+      </c>
+      <c r="D19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" t="s">
+        <v>291</v>
+      </c>
+      <c r="F19" t="s">
+        <v>292</v>
+      </c>
+      <c r="G19" t="s">
+        <v>297</v>
+      </c>
+      <c r="H19" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>94</v>
+      </c>
+      <c r="B20" t="s">
+        <v>93</v>
+      </c>
+      <c r="C20">
+        <v>2013</v>
+      </c>
+      <c r="D20" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" t="s">
+        <v>291</v>
+      </c>
+      <c r="F20" t="s">
+        <v>292</v>
+      </c>
+      <c r="G20" t="s">
+        <v>294</v>
+      </c>
+      <c r="H20" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>98</v>
+      </c>
+      <c r="B21" t="s">
+        <v>97</v>
+      </c>
+      <c r="C21">
+        <v>2013</v>
+      </c>
+      <c r="D21" t="s">
+        <v>20</v>
+      </c>
+      <c r="E21" t="s">
+        <v>291</v>
+      </c>
+      <c r="F21" t="s">
+        <v>292</v>
+      </c>
+      <c r="G21" t="s">
+        <v>294</v>
+      </c>
+      <c r="H21" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>102</v>
+      </c>
+      <c r="B22" t="s">
+        <v>101</v>
+      </c>
+      <c r="C22">
+        <v>2013</v>
+      </c>
+      <c r="D22" t="s">
+        <v>20</v>
+      </c>
+      <c r="E22" t="s">
+        <v>291</v>
+      </c>
+      <c r="F22" t="s">
+        <v>292</v>
+      </c>
+      <c r="G22" t="s">
+        <v>308</v>
+      </c>
+      <c r="H22" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>106</v>
+      </c>
+      <c r="B23" t="s">
+        <v>105</v>
+      </c>
+      <c r="C23">
+        <v>2008</v>
+      </c>
+      <c r="D23" t="s">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>298</v>
+      </c>
+      <c r="F23" t="s">
+        <v>299</v>
+      </c>
+      <c r="G23" t="s">
+        <v>300</v>
+      </c>
+      <c r="H23" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>110</v>
+      </c>
+      <c r="B24" t="s">
+        <v>109</v>
+      </c>
+      <c r="C24">
+        <v>2012</v>
+      </c>
+      <c r="D24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E24" t="s">
+        <v>291</v>
+      </c>
+      <c r="F24" t="s">
+        <v>292</v>
+      </c>
+      <c r="G24" t="s">
+        <v>293</v>
+      </c>
+      <c r="H24" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>114</v>
+      </c>
+      <c r="B25" t="s">
+        <v>113</v>
+      </c>
+      <c r="C25">
+        <v>2012</v>
+      </c>
+      <c r="D25" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25" t="s">
+        <v>291</v>
+      </c>
+      <c r="F25" t="s">
+        <v>292</v>
+      </c>
+      <c r="G25" t="s">
+        <v>297</v>
+      </c>
+      <c r="H25" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>119</v>
+      </c>
+      <c r="B26" t="s">
+        <v>118</v>
+      </c>
+      <c r="C26">
+        <v>2012</v>
+      </c>
+      <c r="D26" t="s">
+        <v>20</v>
+      </c>
+      <c r="E26" t="s">
+        <v>291</v>
+      </c>
+      <c r="F26" t="s">
+        <v>295</v>
+      </c>
+      <c r="G26" t="s">
+        <v>296</v>
+      </c>
+      <c r="H26" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>123</v>
+      </c>
+      <c r="B27" t="s">
+        <v>122</v>
+      </c>
+      <c r="C27">
+        <v>2008</v>
+      </c>
+      <c r="D27" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" t="s">
+        <v>298</v>
+      </c>
+      <c r="F27" t="s">
+        <v>299</v>
+      </c>
+      <c r="G27" t="s">
+        <v>328</v>
+      </c>
+      <c r="H27" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>127</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C28">
+        <v>2008</v>
+      </c>
+      <c r="D28" t="s">
+        <v>20</v>
+      </c>
+      <c r="E28" t="s">
+        <v>298</v>
+      </c>
+      <c r="F28" t="s">
+        <v>301</v>
+      </c>
+      <c r="G28" t="s">
+        <v>305</v>
+      </c>
+      <c r="H28" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>132</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C29">
+        <v>1960</v>
+      </c>
+      <c r="D29" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" t="s">
+        <v>298</v>
+      </c>
+      <c r="F29" t="s">
+        <v>302</v>
+      </c>
+      <c r="G29" t="s">
+        <v>305</v>
+      </c>
+      <c r="H29" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>136</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="C30">
+        <v>2002</v>
+      </c>
+      <c r="D30" t="s">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>291</v>
+      </c>
+      <c r="F30" t="s">
+        <v>303</v>
+      </c>
+      <c r="G30" t="s">
+        <v>305</v>
+      </c>
+      <c r="H30" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>140</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C31">
+        <v>2008</v>
+      </c>
+      <c r="D31" t="s">
+        <v>20</v>
+      </c>
+      <c r="E31" t="s">
+        <v>298</v>
+      </c>
+      <c r="F31" t="s">
+        <v>304</v>
+      </c>
+      <c r="G31" t="s">
+        <v>305</v>
+      </c>
+      <c r="H31" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>144</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C32">
+        <v>2008</v>
+      </c>
+      <c r="D32" t="s">
+        <v>20</v>
+      </c>
+      <c r="E32" t="s">
+        <v>298</v>
+      </c>
+      <c r="F32" t="s">
+        <v>299</v>
+      </c>
+      <c r="G32" t="s">
+        <v>305</v>
+      </c>
+      <c r="H32" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>148</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="C33">
+        <v>2008</v>
+      </c>
+      <c r="D33" t="s">
+        <v>20</v>
+      </c>
+      <c r="E33" t="s">
+        <v>298</v>
+      </c>
+      <c r="F33" t="s">
+        <v>302</v>
+      </c>
+      <c r="G33" t="s">
+        <v>305</v>
+      </c>
+      <c r="H33" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>151</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C34">
+        <v>2008</v>
+      </c>
+      <c r="D34" t="s">
+        <v>20</v>
+      </c>
+      <c r="E34" t="s">
+        <v>298</v>
+      </c>
+      <c r="F34" t="s">
+        <v>301</v>
+      </c>
+      <c r="G34" t="s">
+        <v>305</v>
+      </c>
+      <c r="H34" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>155</v>
+      </c>
+      <c r="B35" t="s">
+        <v>154</v>
+      </c>
+      <c r="C35">
+        <v>2009</v>
+      </c>
+      <c r="D35" t="s">
+        <v>20</v>
+      </c>
+      <c r="E35" t="s">
+        <v>298</v>
+      </c>
+      <c r="F35" t="s">
+        <v>299</v>
+      </c>
+      <c r="G35" t="s">
+        <v>328</v>
+      </c>
+      <c r="H35" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>159</v>
+      </c>
+      <c r="B36" t="s">
+        <v>154</v>
+      </c>
+      <c r="C36">
+        <v>2009</v>
+      </c>
+      <c r="D36" t="s">
+        <v>20</v>
+      </c>
+      <c r="E36" t="s">
+        <v>298</v>
+      </c>
+      <c r="F36" t="s">
+        <v>299</v>
+      </c>
+      <c r="G36" t="s">
+        <v>328</v>
+      </c>
+      <c r="H36" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>162</v>
+      </c>
+      <c r="B37" t="s">
+        <v>154</v>
+      </c>
+      <c r="C37">
+        <v>2009</v>
+      </c>
+      <c r="D37" t="s">
+        <v>20</v>
+      </c>
+      <c r="E37" t="s">
+        <v>298</v>
+      </c>
+      <c r="F37" t="s">
+        <v>299</v>
+      </c>
+      <c r="G37" t="s">
+        <v>328</v>
+      </c>
+      <c r="H37" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>165</v>
+      </c>
+      <c r="B38" t="s">
+        <v>154</v>
+      </c>
+      <c r="C38">
+        <v>2009</v>
+      </c>
+      <c r="D38" t="s">
+        <v>20</v>
+      </c>
+      <c r="E38" t="s">
+        <v>298</v>
+      </c>
+      <c r="F38" t="s">
+        <v>299</v>
+      </c>
+      <c r="G38" t="s">
+        <v>328</v>
+      </c>
+      <c r="H38" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>169</v>
+      </c>
+      <c r="B39" t="s">
+        <v>168</v>
+      </c>
+      <c r="C39">
+        <v>2009</v>
+      </c>
+      <c r="D39" t="s">
+        <v>25</v>
+      </c>
+      <c r="E39" t="s">
+        <v>323</v>
+      </c>
+      <c r="F39" t="s">
+        <v>324</v>
+      </c>
+      <c r="G39" t="s">
+        <v>305</v>
+      </c>
+      <c r="H39" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>172</v>
+      </c>
+      <c r="B40" t="s">
+        <v>171</v>
+      </c>
+      <c r="C40">
+        <v>2009</v>
+      </c>
+      <c r="D40" t="s">
+        <v>25</v>
+      </c>
+      <c r="E40" t="s">
+        <v>336</v>
+      </c>
+      <c r="F40" t="s">
+        <v>338</v>
+      </c>
+      <c r="G40" t="s">
+        <v>305</v>
+      </c>
+      <c r="H40" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>175</v>
+      </c>
+      <c r="B41" t="s">
+        <v>174</v>
+      </c>
+      <c r="C41">
+        <v>2009</v>
+      </c>
+      <c r="D41" t="s">
+        <v>20</v>
+      </c>
+      <c r="E41" t="s">
+        <v>298</v>
+      </c>
+      <c r="F41" t="s">
+        <v>339</v>
+      </c>
+      <c r="G41" t="s">
+        <v>340</v>
+      </c>
+      <c r="H41" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>178</v>
+      </c>
+      <c r="B42" t="s">
+        <v>177</v>
+      </c>
+      <c r="C42">
+        <v>2009</v>
+      </c>
+      <c r="D42" t="s">
+        <v>20</v>
+      </c>
+      <c r="E42" t="s">
+        <v>298</v>
+      </c>
+      <c r="F42" t="s">
+        <v>341</v>
+      </c>
+      <c r="G42" t="s">
+        <v>342</v>
+      </c>
+      <c r="H42" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>181</v>
+      </c>
+      <c r="B43" t="s">
+        <v>180</v>
+      </c>
+      <c r="C43">
+        <v>2009</v>
+      </c>
+      <c r="D43" t="s">
+        <v>20</v>
+      </c>
+      <c r="E43" t="s">
+        <v>298</v>
+      </c>
+      <c r="F43" t="s">
+        <v>343</v>
+      </c>
+      <c r="G43" t="s">
+        <v>344</v>
+      </c>
+      <c r="H43" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>184</v>
+      </c>
+      <c r="B44" t="s">
+        <v>183</v>
+      </c>
+      <c r="C44">
+        <v>2010</v>
+      </c>
+      <c r="D44" t="s">
+        <v>20</v>
+      </c>
+      <c r="E44" t="s">
+        <v>291</v>
+      </c>
+      <c r="F44" t="s">
+        <v>319</v>
+      </c>
+      <c r="G44" t="s">
+        <v>345</v>
+      </c>
+      <c r="H44" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>187</v>
+      </c>
+      <c r="B45" t="s">
+        <v>186</v>
+      </c>
+      <c r="C45">
+        <v>2010</v>
+      </c>
+      <c r="D45" t="s">
+        <v>20</v>
+      </c>
+      <c r="E45" t="s">
+        <v>298</v>
+      </c>
+      <c r="F45" t="s">
+        <v>354</v>
+      </c>
+      <c r="G45" t="s">
+        <v>366</v>
+      </c>
+      <c r="H45" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>190</v>
+      </c>
+      <c r="B46" t="s">
+        <v>189</v>
+      </c>
+      <c r="C46">
+        <v>2008</v>
+      </c>
+      <c r="D46" t="s">
+        <v>20</v>
+      </c>
+      <c r="E46" t="s">
+        <v>298</v>
+      </c>
+      <c r="F46" t="s">
+        <v>304</v>
+      </c>
+      <c r="G46" t="s">
+        <v>360</v>
+      </c>
+      <c r="H46" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>194</v>
+      </c>
+      <c r="B47" t="s">
+        <v>192</v>
+      </c>
+      <c r="C47">
+        <v>2009</v>
+      </c>
+      <c r="D47" t="s">
+        <v>20</v>
+      </c>
+      <c r="E47" t="s">
+        <v>298</v>
+      </c>
+      <c r="F47" t="s">
+        <v>349</v>
+      </c>
+      <c r="G47" t="s">
+        <v>350</v>
+      </c>
+      <c r="H47" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>197</v>
+      </c>
+      <c r="B48" t="s">
+        <v>196</v>
+      </c>
+      <c r="C48">
+        <v>2009</v>
+      </c>
+      <c r="D48" t="s">
+        <v>20</v>
+      </c>
+      <c r="E48" t="s">
+        <v>298</v>
+      </c>
+      <c r="F48" t="s">
+        <v>351</v>
+      </c>
+      <c r="G48" t="s">
+        <v>352</v>
+      </c>
+      <c r="H48" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>200</v>
+      </c>
+      <c r="B49" t="s">
+        <v>199</v>
+      </c>
+      <c r="C49">
+        <v>2008</v>
+      </c>
+      <c r="D49" t="s">
+        <v>20</v>
+      </c>
+      <c r="E49" t="s">
+        <v>298</v>
+      </c>
+      <c r="F49" t="s">
+        <v>348</v>
+      </c>
+      <c r="G49" t="s">
+        <v>361</v>
+      </c>
+      <c r="H49" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>203</v>
+      </c>
+      <c r="B50" t="s">
+        <v>41</v>
+      </c>
+      <c r="C50">
+        <v>2015</v>
+      </c>
+      <c r="D50" t="s">
+        <v>20</v>
+      </c>
+      <c r="E50" t="s">
+        <v>298</v>
+      </c>
+      <c r="F50" t="s">
+        <v>310</v>
+      </c>
+      <c r="G50" t="s">
+        <v>311</v>
+      </c>
+      <c r="H50" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>206</v>
+      </c>
+      <c r="B51" t="s">
+        <v>47</v>
+      </c>
+      <c r="C51">
+        <v>2016</v>
+      </c>
+      <c r="D51" t="s">
+        <v>20</v>
+      </c>
+      <c r="E51" t="s">
+        <v>298</v>
+      </c>
+      <c r="F51" t="s">
+        <v>312</v>
+      </c>
+      <c r="G51" t="s">
+        <v>313</v>
+      </c>
+      <c r="H51" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>210</v>
+      </c>
+      <c r="B52" t="s">
+        <v>209</v>
+      </c>
+      <c r="C52">
+        <v>2009</v>
+      </c>
+      <c r="D52" t="s">
+        <v>25</v>
+      </c>
+      <c r="E52" t="s">
+        <v>335</v>
+      </c>
+      <c r="F52" t="s">
+        <v>337</v>
+      </c>
+      <c r="G52" t="s">
+        <v>305</v>
+      </c>
+      <c r="H52" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>213</v>
+      </c>
+      <c r="B53" t="s">
+        <v>202</v>
+      </c>
+      <c r="C53">
+        <v>2008</v>
+      </c>
+      <c r="D53" t="s">
+        <v>20</v>
+      </c>
+      <c r="E53" t="s">
+        <v>298</v>
+      </c>
+      <c r="F53" t="s">
+        <v>349</v>
+      </c>
+      <c r="G53" t="s">
+        <v>350</v>
+      </c>
+      <c r="H53" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>216</v>
+      </c>
+      <c r="B54" t="s">
+        <v>205</v>
+      </c>
+      <c r="C54">
+        <v>2010</v>
+      </c>
+      <c r="D54" t="s">
+        <v>20</v>
+      </c>
+      <c r="E54" t="s">
+        <v>298</v>
+      </c>
+      <c r="F54" t="s">
+        <v>354</v>
+      </c>
+      <c r="G54" t="s">
+        <v>365</v>
+      </c>
+      <c r="H54" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>219</v>
+      </c>
+      <c r="B55" t="s">
+        <v>208</v>
+      </c>
+      <c r="C55">
+        <v>2010</v>
+      </c>
+      <c r="D55" t="s">
+        <v>20</v>
+      </c>
+      <c r="E55" t="s">
+        <v>298</v>
+      </c>
+      <c r="F55" t="s">
+        <v>355</v>
+      </c>
+      <c r="G55" t="s">
+        <v>367</v>
+      </c>
+      <c r="H55" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>221</v>
+      </c>
+      <c r="B56" t="s">
+        <v>212</v>
+      </c>
+      <c r="C56">
+        <v>2009</v>
+      </c>
+      <c r="D56" t="s">
+        <v>20</v>
+      </c>
+      <c r="E56" t="s">
+        <v>298</v>
+      </c>
+      <c r="F56" t="s">
+        <v>299</v>
+      </c>
+      <c r="G56" t="s">
+        <v>353</v>
+      </c>
+      <c r="H56" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>224</v>
+      </c>
+      <c r="B57" t="s">
+        <v>134</v>
+      </c>
+      <c r="C57">
+        <v>2010</v>
+      </c>
+      <c r="D57" t="s">
+        <v>20</v>
+      </c>
+      <c r="E57" t="s">
+        <v>298</v>
+      </c>
+      <c r="F57" t="s">
+        <v>304</v>
+      </c>
+      <c r="G57" t="s">
+        <v>364</v>
+      </c>
+      <c r="H57" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>227</v>
+      </c>
+      <c r="B58" t="s">
+        <v>138</v>
+      </c>
+      <c r="C58">
+        <v>2010</v>
+      </c>
+      <c r="D58" t="s">
+        <v>20</v>
+      </c>
+      <c r="E58" t="s">
+        <v>291</v>
+      </c>
+      <c r="F58" t="s">
+        <v>319</v>
+      </c>
+      <c r="G58" t="s">
+        <v>305</v>
+      </c>
+      <c r="H58" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>230</v>
+      </c>
+      <c r="B59" t="s">
+        <v>142</v>
+      </c>
+      <c r="C59">
+        <v>2010</v>
+      </c>
+      <c r="D59" t="s">
+        <v>20</v>
+      </c>
+      <c r="E59" t="s">
+        <v>298</v>
+      </c>
+      <c r="F59" t="s">
+        <v>354</v>
+      </c>
+      <c r="G59" t="s">
+        <v>368</v>
+      </c>
+      <c r="H59" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>234</v>
+      </c>
+      <c r="B60" t="s">
+        <v>150</v>
+      </c>
+      <c r="C60">
+        <v>2016</v>
+      </c>
+      <c r="D60" t="s">
+        <v>236</v>
+      </c>
+      <c r="E60" t="s">
+        <v>237</v>
+      </c>
+      <c r="F60" t="s">
+        <v>305</v>
+      </c>
+      <c r="G60" t="s">
+        <v>237</v>
+      </c>
+      <c r="H60" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>238</v>
+      </c>
+      <c r="B61" t="s">
+        <v>153</v>
+      </c>
+      <c r="C61">
+        <v>2016</v>
+      </c>
+      <c r="D61" t="s">
+        <v>236</v>
+      </c>
+      <c r="E61" t="s">
+        <v>237</v>
+      </c>
+      <c r="F61" t="s">
+        <v>305</v>
+      </c>
+      <c r="G61" t="s">
+        <v>237</v>
+      </c>
+      <c r="H61" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>241</v>
+      </c>
+      <c r="B62" t="s">
+        <v>157</v>
+      </c>
+      <c r="C62">
+        <v>2012</v>
+      </c>
+      <c r="D62" t="s">
+        <v>20</v>
+      </c>
+      <c r="E62" t="s">
+        <v>291</v>
+      </c>
+      <c r="F62" t="s">
+        <v>292</v>
+      </c>
+      <c r="G62" t="s">
+        <v>297</v>
+      </c>
+      <c r="H62" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>244</v>
+      </c>
+      <c r="B63" t="s">
+        <v>161</v>
+      </c>
+      <c r="C63">
+        <v>2012</v>
+      </c>
+      <c r="D63" t="s">
+        <v>20</v>
+      </c>
+      <c r="E63" t="s">
+        <v>298</v>
+      </c>
+      <c r="F63" t="s">
+        <v>359</v>
+      </c>
+      <c r="G63" t="s">
+        <v>374</v>
+      </c>
+      <c r="H63" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>247</v>
+      </c>
+      <c r="B64" t="s">
+        <v>246</v>
+      </c>
+      <c r="C64">
+        <v>2011</v>
+      </c>
+      <c r="D64" t="s">
+        <v>20</v>
+      </c>
+      <c r="E64" t="s">
+        <v>298</v>
+      </c>
+      <c r="F64" t="s">
+        <v>351</v>
+      </c>
+      <c r="G64" t="s">
+        <v>371</v>
+      </c>
+      <c r="H64" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>249</v>
+      </c>
+      <c r="B65" t="s">
+        <v>164</v>
+      </c>
+      <c r="C65">
+        <v>2011</v>
+      </c>
+      <c r="D65" t="s">
+        <v>20</v>
+      </c>
+      <c r="E65" t="s">
+        <v>298</v>
+      </c>
+      <c r="F65" t="s">
+        <v>354</v>
+      </c>
+      <c r="G65" t="s">
+        <v>366</v>
+      </c>
+      <c r="H65" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>252</v>
+      </c>
+      <c r="B66" t="s">
+        <v>251</v>
+      </c>
+      <c r="C66">
+        <v>2011</v>
+      </c>
+      <c r="D66" t="s">
+        <v>20</v>
+      </c>
+      <c r="E66" t="s">
+        <v>298</v>
+      </c>
+      <c r="F66" t="s">
+        <v>356</v>
+      </c>
+      <c r="G66" t="s">
+        <v>370</v>
+      </c>
+      <c r="H66" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>255</v>
+      </c>
+      <c r="B67" t="s">
+        <v>254</v>
+      </c>
+      <c r="C67">
+        <v>2011</v>
+      </c>
+      <c r="D67" t="s">
+        <v>20</v>
+      </c>
+      <c r="E67" t="s">
+        <v>298</v>
+      </c>
+      <c r="F67" t="s">
+        <v>356</v>
+      </c>
+      <c r="G67" t="s">
+        <v>369</v>
+      </c>
+      <c r="H67" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>259</v>
+      </c>
+      <c r="B68" t="s">
+        <v>258</v>
+      </c>
+      <c r="C68">
+        <v>2012</v>
+      </c>
+      <c r="D68" t="s">
+        <v>20</v>
+      </c>
+      <c r="E68" t="s">
+        <v>298</v>
+      </c>
+      <c r="F68" t="s">
+        <v>358</v>
+      </c>
+      <c r="G68" t="s">
+        <v>373</v>
+      </c>
+      <c r="H68" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>261</v>
+      </c>
+      <c r="B69" t="s">
+        <v>215</v>
+      </c>
+      <c r="C69">
+        <v>2011</v>
+      </c>
+      <c r="D69" t="s">
+        <v>20</v>
+      </c>
+      <c r="E69" t="s">
+        <v>298</v>
+      </c>
+      <c r="F69" t="s">
+        <v>357</v>
+      </c>
+      <c r="G69" t="s">
+        <v>372</v>
+      </c>
+      <c r="H69" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>265</v>
+      </c>
+      <c r="B70" t="s">
+        <v>264</v>
+      </c>
+      <c r="C70">
+        <v>2011</v>
+      </c>
+      <c r="D70" t="s">
+        <v>25</v>
+      </c>
+      <c r="E70" t="s">
+        <v>268</v>
+      </c>
+      <c r="F70" t="s">
+        <v>305</v>
+      </c>
+      <c r="G70" t="s">
+        <v>305</v>
+      </c>
+      <c r="H70" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>270</v>
+      </c>
+      <c r="B71" t="s">
+        <v>269</v>
+      </c>
+      <c r="C71">
+        <v>2009</v>
+      </c>
+      <c r="D71" t="s">
+        <v>25</v>
+      </c>
+      <c r="E71" t="s">
+        <v>346</v>
+      </c>
+      <c r="F71" t="s">
+        <v>363</v>
+      </c>
+      <c r="G71" t="s">
+        <v>362</v>
+      </c>
+      <c r="H71" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>274</v>
+      </c>
+      <c r="B72" t="s">
+        <v>273</v>
+      </c>
+      <c r="C72">
+        <v>2014</v>
+      </c>
+      <c r="D72" t="s">
+        <v>20</v>
+      </c>
+      <c r="E72" t="s">
+        <v>291</v>
+      </c>
+      <c r="F72" t="s">
+        <v>319</v>
+      </c>
+      <c r="G72" t="s">
+        <v>334</v>
+      </c>
+      <c r="H72" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>278</v>
+      </c>
+      <c r="B73" t="s">
+        <v>277</v>
+      </c>
+      <c r="C73">
+        <v>2013</v>
+      </c>
+      <c r="D73" t="s">
+        <v>20</v>
+      </c>
+      <c r="E73" t="s">
+        <v>291</v>
+      </c>
+      <c r="F73" t="s">
+        <v>322</v>
+      </c>
+      <c r="G73" t="s">
+        <v>333</v>
+      </c>
+      <c r="H73" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>282</v>
+      </c>
+      <c r="B74" t="s">
+        <v>281</v>
+      </c>
+      <c r="C74">
+        <v>2012</v>
+      </c>
+      <c r="D74" t="s">
+        <v>20</v>
+      </c>
+      <c r="E74" t="s">
+        <v>291</v>
+      </c>
+      <c r="F74" t="s">
+        <v>292</v>
+      </c>
+      <c r="G74" t="s">
+        <v>332</v>
+      </c>
+      <c r="H74" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>286</v>
+      </c>
+      <c r="B75" t="s">
+        <v>285</v>
+      </c>
+      <c r="C75">
+        <v>2012</v>
+      </c>
+      <c r="D75" t="s">
+        <v>20</v>
+      </c>
+      <c r="E75" t="s">
+        <v>291</v>
+      </c>
+      <c r="F75" t="s">
+        <v>292</v>
+      </c>
+      <c r="G75" t="s">
+        <v>297</v>
+      </c>
+      <c r="H75" t="s">
+        <v>433</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="19" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>